<commit_message>
add method MS and change required binding to extensible (#79) 4c51a5196195117c72ed8880a5e96245f4854ddf
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
+++ b/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$116</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4914" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4491" uniqueCount="696">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-28T12:14:54+00:00</t>
+    <t>2023-11-28T12:15:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1792,39 +1792,6 @@
   </si>
   <si>
     <t>methodCode</t>
-  </si>
-  <si>
-    <t>Observation.method.id</t>
-  </si>
-  <si>
-    <t>Observation.method.extension</t>
-  </si>
-  <si>
-    <t>Observation.method.coding</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.id</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.extension</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.system</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.version</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.code</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.display</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.userSelected</t>
-  </si>
-  <si>
-    <t>Observation.method.text</t>
   </si>
   <si>
     <t>Observation.specimen</t>
@@ -2537,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP127"/>
+  <dimension ref="A1:AP116"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.58984375" customWidth="true" bestFit="true"/>
@@ -2564,7 +2531,7 @@
     <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="109.11328125" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="111.65625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
@@ -13718,7 +13685,7 @@
         <v>91</v>
       </c>
       <c r="H93" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I93" t="s" s="2">
         <v>80</v>
@@ -13764,11 +13731,9 @@
         <v>80</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="Y93" t="s" s="2">
-        <v>569</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="Y93" s="2"/>
       <c r="Z93" t="s" s="2">
         <v>569</v>
       </c>
@@ -13849,15 +13814,17 @@
         <v>80</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>107</v>
+        <v>573</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>108</v>
+        <v>574</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N94" s="2"/>
+        <v>575</v>
+      </c>
+      <c r="N94" t="s" s="2">
+        <v>576</v>
+      </c>
       <c r="O94" s="2"/>
       <c r="P94" t="s" s="2">
         <v>80</v>
@@ -13906,7 +13873,7 @@
         <v>80</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>110</v>
+        <v>572</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
@@ -13915,47 +13882,47 @@
         <v>91</v>
       </c>
       <c r="AI94" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>80</v>
+        <v>233</v>
       </c>
       <c r="AK94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL94" t="s" s="2">
-        <v>80</v>
+        <v>577</v>
       </c>
       <c r="AM94" t="s" s="2">
-        <v>80</v>
+        <v>578</v>
       </c>
       <c r="AN94" t="s" s="2">
-        <v>111</v>
+        <v>579</v>
       </c>
       <c r="AO94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP94" t="s" s="2">
-        <v>80</v>
+        <v>580</v>
       </c>
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E95" s="2"/>
       <c r="F95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H95" t="s" s="2">
         <v>80</v>
@@ -13967,16 +13934,16 @@
         <v>80</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>114</v>
+        <v>582</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>115</v>
+        <v>583</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>116</v>
+        <v>584</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>117</v>
+        <v>585</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -14014,57 +13981,57 @@
         <v>80</v>
       </c>
       <c r="AB95" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC95" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE95" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>121</v>
+        <v>581</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH95" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI95" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>122</v>
+        <v>233</v>
       </c>
       <c r="AK95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>80</v>
+        <v>586</v>
       </c>
       <c r="AM95" t="s" s="2">
-        <v>80</v>
+        <v>587</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>105</v>
+        <v>588</v>
       </c>
       <c r="AO95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP95" t="s" s="2">
-        <v>80</v>
+        <v>589</v>
       </c>
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -14084,22 +14051,22 @@
         <v>80</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K96" t="s" s="2">
-        <v>147</v>
+        <v>591</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>279</v>
+        <v>592</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>280</v>
+        <v>593</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>281</v>
+        <v>594</v>
       </c>
       <c r="O96" t="s" s="2">
-        <v>282</v>
+        <v>595</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>80</v>
@@ -14148,7 +14115,7 @@
         <v>80</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>283</v>
+        <v>590</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>78</v>
@@ -14160,7 +14127,7 @@
         <v>103</v>
       </c>
       <c r="AJ96" t="s" s="2">
-        <v>104</v>
+        <v>596</v>
       </c>
       <c r="AK96" t="s" s="2">
         <v>80</v>
@@ -14169,10 +14136,10 @@
         <v>80</v>
       </c>
       <c r="AM96" t="s" s="2">
-        <v>284</v>
+        <v>597</v>
       </c>
       <c r="AN96" t="s" s="2">
-        <v>285</v>
+        <v>598</v>
       </c>
       <c r="AO96" t="s" s="2">
         <v>80</v>
@@ -14183,10 +14150,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -14301,10 +14268,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>576</v>
+        <v>600</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>576</v>
+        <v>600</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -14421,45 +14388,45 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
-        <v>80</v>
+        <v>602</v>
       </c>
       <c r="E99" s="2"/>
       <c r="F99" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H99" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I99" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J99" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>292</v>
+        <v>603</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>293</v>
+        <v>604</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>294</v>
+        <v>117</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>295</v>
+        <v>215</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>80</v>
@@ -14508,19 +14475,19 @@
         <v>80</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>297</v>
+        <v>605</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH99" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI99" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ99" t="s" s="2">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="AK99" t="s" s="2">
         <v>80</v>
@@ -14529,10 +14496,10 @@
         <v>80</v>
       </c>
       <c r="AM99" t="s" s="2">
-        <v>298</v>
+        <v>80</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>299</v>
+        <v>105</v>
       </c>
       <c r="AO99" t="s" s="2">
         <v>80</v>
@@ -14543,10 +14510,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>578</v>
+        <v>606</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>578</v>
+        <v>606</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -14566,19 +14533,19 @@
         <v>80</v>
       </c>
       <c r="J100" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>107</v>
+        <v>607</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>302</v>
+        <v>608</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>303</v>
+        <v>609</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>304</v>
+        <v>610</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -14628,7 +14595,7 @@
         <v>80</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>305</v>
+        <v>606</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>78</v>
@@ -14637,10 +14604,10 @@
         <v>91</v>
       </c>
       <c r="AI100" t="s" s="2">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>104</v>
+        <v>612</v>
       </c>
       <c r="AK100" t="s" s="2">
         <v>80</v>
@@ -14649,10 +14616,10 @@
         <v>80</v>
       </c>
       <c r="AM100" t="s" s="2">
-        <v>306</v>
+        <v>613</v>
       </c>
       <c r="AN100" t="s" s="2">
-        <v>307</v>
+        <v>614</v>
       </c>
       <c r="AO100" t="s" s="2">
         <v>80</v>
@@ -14663,10 +14630,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>579</v>
+        <v>615</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>579</v>
+        <v>615</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14674,7 +14641,7 @@
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G101" t="s" s="2">
         <v>91</v>
@@ -14686,23 +14653,21 @@
         <v>80</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>171</v>
+        <v>607</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>310</v>
+        <v>616</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>311</v>
+        <v>617</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="O101" t="s" s="2">
-        <v>313</v>
-      </c>
+        <v>610</v>
+      </c>
+      <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
         <v>80</v>
       </c>
@@ -14750,7 +14715,7 @@
         <v>80</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>315</v>
+        <v>615</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>78</v>
@@ -14759,10 +14724,10 @@
         <v>91</v>
       </c>
       <c r="AI101" t="s" s="2">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>104</v>
+        <v>612</v>
       </c>
       <c r="AK101" t="s" s="2">
         <v>80</v>
@@ -14771,10 +14736,10 @@
         <v>80</v>
       </c>
       <c r="AM101" t="s" s="2">
-        <v>316</v>
+        <v>613</v>
       </c>
       <c r="AN101" t="s" s="2">
-        <v>317</v>
+        <v>618</v>
       </c>
       <c r="AO101" t="s" s="2">
         <v>80</v>
@@ -14785,10 +14750,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>580</v>
+        <v>619</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>580</v>
+        <v>619</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14808,22 +14773,22 @@
         <v>80</v>
       </c>
       <c r="J102" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>107</v>
+        <v>260</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>320</v>
+        <v>620</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>321</v>
+        <v>621</v>
       </c>
       <c r="N102" t="s" s="2">
-        <v>312</v>
+        <v>622</v>
       </c>
       <c r="O102" t="s" s="2">
-        <v>322</v>
+        <v>623</v>
       </c>
       <c r="P102" t="s" s="2">
         <v>80</v>
@@ -14848,13 +14813,13 @@
         <v>80</v>
       </c>
       <c r="X102" t="s" s="2">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="Y102" t="s" s="2">
-        <v>80</v>
+        <v>624</v>
       </c>
       <c r="Z102" t="s" s="2">
-        <v>80</v>
+        <v>625</v>
       </c>
       <c r="AA102" t="s" s="2">
         <v>80</v>
@@ -14872,7 +14837,7 @@
         <v>80</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>323</v>
+        <v>619</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>78</v>
@@ -14890,13 +14855,13 @@
         <v>80</v>
       </c>
       <c r="AL102" t="s" s="2">
-        <v>80</v>
+        <v>626</v>
       </c>
       <c r="AM102" t="s" s="2">
-        <v>324</v>
+        <v>627</v>
       </c>
       <c r="AN102" t="s" s="2">
-        <v>325</v>
+        <v>534</v>
       </c>
       <c r="AO102" t="s" s="2">
         <v>80</v>
@@ -14907,10 +14872,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>581</v>
+        <v>628</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>581</v>
+        <v>628</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14921,7 +14886,7 @@
         <v>78</v>
       </c>
       <c r="G103" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H103" t="s" s="2">
         <v>80</v>
@@ -14930,22 +14895,22 @@
         <v>80</v>
       </c>
       <c r="J103" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>328</v>
+        <v>260</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>329</v>
+        <v>629</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>330</v>
+        <v>630</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>331</v>
+        <v>631</v>
       </c>
       <c r="O103" t="s" s="2">
-        <v>332</v>
+        <v>632</v>
       </c>
       <c r="P103" t="s" s="2">
         <v>80</v>
@@ -14970,13 +14935,13 @@
         <v>80</v>
       </c>
       <c r="X103" t="s" s="2">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="Y103" t="s" s="2">
-        <v>80</v>
+        <v>633</v>
       </c>
       <c r="Z103" t="s" s="2">
-        <v>80</v>
+        <v>634</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>80</v>
@@ -14994,13 +14959,13 @@
         <v>80</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>333</v>
+        <v>628</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH103" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI103" t="s" s="2">
         <v>103</v>
@@ -15012,13 +14977,13 @@
         <v>80</v>
       </c>
       <c r="AL103" t="s" s="2">
-        <v>80</v>
+        <v>626</v>
       </c>
       <c r="AM103" t="s" s="2">
-        <v>334</v>
+        <v>627</v>
       </c>
       <c r="AN103" t="s" s="2">
-        <v>335</v>
+        <v>534</v>
       </c>
       <c r="AO103" t="s" s="2">
         <v>80</v>
@@ -15029,10 +14994,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>582</v>
+        <v>635</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>582</v>
+        <v>635</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -15052,22 +15017,22 @@
         <v>80</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K104" t="s" s="2">
-        <v>107</v>
+        <v>636</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>338</v>
+        <v>637</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>339</v>
+        <v>638</v>
       </c>
       <c r="N104" t="s" s="2">
-        <v>340</v>
+        <v>639</v>
       </c>
       <c r="O104" t="s" s="2">
-        <v>341</v>
+        <v>640</v>
       </c>
       <c r="P104" t="s" s="2">
         <v>80</v>
@@ -15116,7 +15081,7 @@
         <v>80</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>342</v>
+        <v>635</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>78</v>
@@ -15128,7 +15093,7 @@
         <v>103</v>
       </c>
       <c r="AJ104" t="s" s="2">
-        <v>104</v>
+        <v>641</v>
       </c>
       <c r="AK104" t="s" s="2">
         <v>80</v>
@@ -15137,10 +15102,10 @@
         <v>80</v>
       </c>
       <c r="AM104" t="s" s="2">
-        <v>343</v>
+        <v>642</v>
       </c>
       <c r="AN104" t="s" s="2">
-        <v>344</v>
+        <v>643</v>
       </c>
       <c r="AO104" t="s" s="2">
         <v>80</v>
@@ -15151,10 +15116,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -15177,16 +15142,16 @@
         <v>80</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>584</v>
+        <v>107</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>585</v>
+        <v>645</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>586</v>
+        <v>646</v>
       </c>
       <c r="N105" t="s" s="2">
-        <v>587</v>
+        <v>312</v>
       </c>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
@@ -15236,7 +15201,7 @@
         <v>80</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>78</v>
@@ -15248,33 +15213,33 @@
         <v>103</v>
       </c>
       <c r="AJ105" t="s" s="2">
-        <v>233</v>
+        <v>104</v>
       </c>
       <c r="AK105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL105" t="s" s="2">
-        <v>588</v>
+        <v>80</v>
       </c>
       <c r="AM105" t="s" s="2">
-        <v>589</v>
+        <v>613</v>
       </c>
       <c r="AN105" t="s" s="2">
-        <v>590</v>
+        <v>647</v>
       </c>
       <c r="AO105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP105" t="s" s="2">
-        <v>591</v>
+        <v>80</v>
       </c>
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -15285,7 +15250,7 @@
         <v>78</v>
       </c>
       <c r="G106" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H106" t="s" s="2">
         <v>80</v>
@@ -15294,19 +15259,19 @@
         <v>80</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K106" t="s" s="2">
-        <v>593</v>
+        <v>649</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>594</v>
+        <v>650</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>595</v>
+        <v>651</v>
       </c>
       <c r="N106" t="s" s="2">
-        <v>596</v>
+        <v>652</v>
       </c>
       <c r="O106" s="2"/>
       <c r="P106" t="s" s="2">
@@ -15356,13 +15321,13 @@
         <v>80</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH106" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI106" t="s" s="2">
         <v>103</v>
@@ -15374,27 +15339,27 @@
         <v>80</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>597</v>
+        <v>80</v>
       </c>
       <c r="AM106" t="s" s="2">
-        <v>598</v>
+        <v>653</v>
       </c>
       <c r="AN106" t="s" s="2">
-        <v>599</v>
+        <v>654</v>
       </c>
       <c r="AO106" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP106" t="s" s="2">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -15414,23 +15379,21 @@
         <v>80</v>
       </c>
       <c r="J107" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>602</v>
+        <v>656</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>603</v>
+        <v>657</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>604</v>
+        <v>658</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O107" t="s" s="2">
-        <v>606</v>
-      </c>
+        <v>659</v>
+      </c>
+      <c r="O107" s="2"/>
       <c r="P107" t="s" s="2">
         <v>80</v>
       </c>
@@ -15478,7 +15441,7 @@
         <v>80</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>78</v>
@@ -15490,7 +15453,7 @@
         <v>103</v>
       </c>
       <c r="AJ107" t="s" s="2">
-        <v>607</v>
+        <v>233</v>
       </c>
       <c r="AK107" t="s" s="2">
         <v>80</v>
@@ -15499,10 +15462,10 @@
         <v>80</v>
       </c>
       <c r="AM107" t="s" s="2">
-        <v>608</v>
+        <v>653</v>
       </c>
       <c r="AN107" t="s" s="2">
-        <v>609</v>
+        <v>660</v>
       </c>
       <c r="AO107" t="s" s="2">
         <v>80</v>
@@ -15513,10 +15476,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -15527,28 +15490,32 @@
         <v>78</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H108" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I108" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J108" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>107</v>
+        <v>591</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>108</v>
+        <v>662</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N108" s="2"/>
-      <c r="O108" s="2"/>
+        <v>662</v>
+      </c>
+      <c r="N108" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="O108" t="s" s="2">
+        <v>664</v>
+      </c>
       <c r="P108" t="s" s="2">
         <v>80</v>
       </c>
@@ -15596,19 +15563,19 @@
         <v>80</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>110</v>
+        <v>661</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH108" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI108" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ108" t="s" s="2">
-        <v>80</v>
+        <v>665</v>
       </c>
       <c r="AK108" t="s" s="2">
         <v>80</v>
@@ -15617,10 +15584,10 @@
         <v>80</v>
       </c>
       <c r="AM108" t="s" s="2">
-        <v>80</v>
+        <v>666</v>
       </c>
       <c r="AN108" t="s" s="2">
-        <v>111</v>
+        <v>667</v>
       </c>
       <c r="AO108" t="s" s="2">
         <v>80</v>
@@ -15631,21 +15598,21 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>611</v>
+        <v>668</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>611</v>
+        <v>668</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E109" s="2"/>
       <c r="F109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H109" t="s" s="2">
         <v>80</v>
@@ -15657,17 +15624,15 @@
         <v>80</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N109" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N109" s="2"/>
       <c r="O109" s="2"/>
       <c r="P109" t="s" s="2">
         <v>80</v>
@@ -15704,31 +15669,31 @@
         <v>80</v>
       </c>
       <c r="AB109" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC109" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD109" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE109" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH109" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI109" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ109" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK109" t="s" s="2">
         <v>80</v>
@@ -15740,7 +15705,7 @@
         <v>80</v>
       </c>
       <c r="AN109" t="s" s="2">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="AO109" t="s" s="2">
         <v>80</v>
@@ -15751,14 +15716,14 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>612</v>
+        <v>669</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>612</v>
+        <v>669</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
-        <v>613</v>
+        <v>113</v>
       </c>
       <c r="E110" s="2"/>
       <c r="F110" t="s" s="2">
@@ -15771,26 +15736,24 @@
         <v>80</v>
       </c>
       <c r="I110" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J110" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K110" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>614</v>
+        <v>115</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>615</v>
+        <v>116</v>
       </c>
       <c r="N110" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O110" t="s" s="2">
-        <v>215</v>
-      </c>
+      <c r="O110" s="2"/>
       <c r="P110" t="s" s="2">
         <v>80</v>
       </c>
@@ -15826,19 +15789,19 @@
         <v>80</v>
       </c>
       <c r="AB110" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC110" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE110" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>616</v>
+        <v>121</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>78</v>
@@ -15873,44 +15836,46 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>617</v>
+        <v>670</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>617</v>
+        <v>670</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
-        <v>80</v>
+        <v>602</v>
       </c>
       <c r="E111" s="2"/>
       <c r="F111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G111" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H111" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I111" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J111" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>618</v>
+        <v>114</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>619</v>
+        <v>603</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>620</v>
+        <v>604</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="O111" s="2"/>
+        <v>117</v>
+      </c>
+      <c r="O111" t="s" s="2">
+        <v>215</v>
+      </c>
       <c r="P111" t="s" s="2">
         <v>80</v>
       </c>
@@ -15958,19 +15923,19 @@
         <v>80</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH111" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI111" t="s" s="2">
-        <v>622</v>
+        <v>103</v>
       </c>
       <c r="AJ111" t="s" s="2">
-        <v>623</v>
+        <v>122</v>
       </c>
       <c r="AK111" t="s" s="2">
         <v>80</v>
@@ -15979,10 +15944,10 @@
         <v>80</v>
       </c>
       <c r="AM111" t="s" s="2">
-        <v>624</v>
+        <v>80</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>625</v>
+        <v>105</v>
       </c>
       <c r="AO111" t="s" s="2">
         <v>80</v>
@@ -15993,10 +15958,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -16004,33 +15969,35 @@
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H112" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J112" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>618</v>
+        <v>260</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>628</v>
+        <v>673</v>
       </c>
       <c r="N112" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="O112" s="2"/>
+        <v>674</v>
+      </c>
+      <c r="O112" t="s" s="2">
+        <v>675</v>
+      </c>
       <c r="P112" t="s" s="2">
         <v>80</v>
       </c>
@@ -16054,13 +16021,13 @@
         <v>80</v>
       </c>
       <c r="X112" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="Y112" t="s" s="2">
-        <v>80</v>
+        <v>351</v>
       </c>
       <c r="Z112" t="s" s="2">
-        <v>80</v>
+        <v>352</v>
       </c>
       <c r="AA112" t="s" s="2">
         <v>80</v>
@@ -16078,34 +16045,34 @@
         <v>80</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="AG112" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="AH112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="AI112" t="s" s="2">
-        <v>622</v>
+        <v>103</v>
       </c>
       <c r="AJ112" t="s" s="2">
-        <v>623</v>
+        <v>104</v>
       </c>
       <c r="AK112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>80</v>
+        <v>676</v>
       </c>
       <c r="AM112" t="s" s="2">
-        <v>624</v>
+        <v>355</v>
       </c>
       <c r="AN112" t="s" s="2">
-        <v>629</v>
+        <v>356</v>
       </c>
       <c r="AO112" t="s" s="2">
-        <v>80</v>
+        <v>357</v>
       </c>
       <c r="AP112" t="s" s="2">
         <v>80</v>
@@ -16113,10 +16080,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -16130,28 +16097,28 @@
         <v>91</v>
       </c>
       <c r="H113" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J113" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>260</v>
+        <v>678</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>631</v>
+        <v>679</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>632</v>
+        <v>680</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>633</v>
+        <v>681</v>
       </c>
       <c r="O113" t="s" s="2">
-        <v>634</v>
+        <v>442</v>
       </c>
       <c r="P113" t="s" s="2">
         <v>80</v>
@@ -16176,13 +16143,13 @@
         <v>80</v>
       </c>
       <c r="X113" t="s" s="2">
-        <v>175</v>
+        <v>251</v>
       </c>
       <c r="Y113" t="s" s="2">
-        <v>635</v>
+        <v>682</v>
       </c>
       <c r="Z113" t="s" s="2">
-        <v>636</v>
+        <v>683</v>
       </c>
       <c r="AA113" t="s" s="2">
         <v>80</v>
@@ -16200,7 +16167,7 @@
         <v>80</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
@@ -16209,7 +16176,7 @@
         <v>91</v>
       </c>
       <c r="AI113" t="s" s="2">
-        <v>103</v>
+        <v>684</v>
       </c>
       <c r="AJ113" t="s" s="2">
         <v>104</v>
@@ -16218,27 +16185,27 @@
         <v>80</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>637</v>
+        <v>685</v>
       </c>
       <c r="AM113" t="s" s="2">
-        <v>638</v>
+        <v>447</v>
       </c>
       <c r="AN113" t="s" s="2">
-        <v>534</v>
+        <v>448</v>
       </c>
       <c r="AO113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP113" t="s" s="2">
-        <v>80</v>
+        <v>449</v>
       </c>
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -16249,10 +16216,10 @@
         <v>78</v>
       </c>
       <c r="G114" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H114" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I114" t="s" s="2">
         <v>80</v>
@@ -16264,16 +16231,16 @@
         <v>260</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>640</v>
+        <v>687</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>641</v>
+        <v>688</v>
       </c>
       <c r="N114" t="s" s="2">
-        <v>642</v>
+        <v>689</v>
       </c>
       <c r="O114" t="s" s="2">
-        <v>643</v>
+        <v>509</v>
       </c>
       <c r="P114" t="s" s="2">
         <v>80</v>
@@ -16298,13 +16265,13 @@
         <v>80</v>
       </c>
       <c r="X114" t="s" s="2">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="Y114" t="s" s="2">
-        <v>644</v>
+        <v>510</v>
       </c>
       <c r="Z114" t="s" s="2">
-        <v>645</v>
+        <v>511</v>
       </c>
       <c r="AA114" t="s" s="2">
         <v>80</v>
@@ -16322,16 +16289,16 @@
         <v>80</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH114" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI114" t="s" s="2">
-        <v>103</v>
+        <v>690</v>
       </c>
       <c r="AJ114" t="s" s="2">
         <v>104</v>
@@ -16340,13 +16307,13 @@
         <v>80</v>
       </c>
       <c r="AL114" t="s" s="2">
-        <v>637</v>
+        <v>80</v>
       </c>
       <c r="AM114" t="s" s="2">
-        <v>638</v>
+        <v>105</v>
       </c>
       <c r="AN114" t="s" s="2">
-        <v>534</v>
+        <v>513</v>
       </c>
       <c r="AO114" t="s" s="2">
         <v>80</v>
@@ -16357,21 +16324,21 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
-        <v>80</v>
+        <v>526</v>
       </c>
       <c r="E115" s="2"/>
       <c r="F115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G115" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H115" t="s" s="2">
         <v>80</v>
@@ -16383,19 +16350,19 @@
         <v>80</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>647</v>
+        <v>260</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>648</v>
+        <v>527</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>649</v>
+        <v>528</v>
       </c>
       <c r="N115" t="s" s="2">
-        <v>650</v>
+        <v>529</v>
       </c>
       <c r="O115" t="s" s="2">
-        <v>651</v>
+        <v>530</v>
       </c>
       <c r="P115" t="s" s="2">
         <v>80</v>
@@ -16420,13 +16387,13 @@
         <v>80</v>
       </c>
       <c r="X115" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="Y115" t="s" s="2">
-        <v>80</v>
+        <v>692</v>
       </c>
       <c r="Z115" t="s" s="2">
-        <v>80</v>
+        <v>531</v>
       </c>
       <c r="AA115" t="s" s="2">
         <v>80</v>
@@ -16444,45 +16411,45 @@
         <v>80</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH115" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI115" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ115" t="s" s="2">
-        <v>652</v>
+        <v>104</v>
       </c>
       <c r="AK115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>80</v>
+        <v>532</v>
       </c>
       <c r="AM115" t="s" s="2">
-        <v>653</v>
+        <v>533</v>
       </c>
       <c r="AN115" t="s" s="2">
-        <v>654</v>
+        <v>534</v>
       </c>
       <c r="AO115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP115" t="s" s="2">
-        <v>80</v>
+        <v>535</v>
       </c>
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -16493,7 +16460,7 @@
         <v>78</v>
       </c>
       <c r="G116" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H116" t="s" s="2">
         <v>80</v>
@@ -16505,18 +16472,20 @@
         <v>80</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>656</v>
+        <v>694</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>657</v>
+        <v>695</v>
       </c>
       <c r="N116" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="O116" s="2"/>
+        <v>594</v>
+      </c>
+      <c r="O116" t="s" s="2">
+        <v>595</v>
+      </c>
       <c r="P116" t="s" s="2">
         <v>80</v>
       </c>
@@ -16564,19 +16533,19 @@
         <v>80</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH116" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI116" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ116" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK116" t="s" s="2">
         <v>80</v>
@@ -16585,1352 +16554,20 @@
         <v>80</v>
       </c>
       <c r="AM116" t="s" s="2">
-        <v>624</v>
+        <v>597</v>
       </c>
       <c r="AN116" t="s" s="2">
-        <v>658</v>
+        <v>598</v>
       </c>
       <c r="AO116" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP116" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="117" hidden="true">
-      <c r="A117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="B117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="C117" s="2"/>
-      <c r="D117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E117" s="2"/>
-      <c r="F117" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G117" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J117" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K117" t="s" s="2">
-        <v>660</v>
-      </c>
-      <c r="L117" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="M117" t="s" s="2">
-        <v>662</v>
-      </c>
-      <c r="N117" t="s" s="2">
-        <v>663</v>
-      </c>
-      <c r="O117" s="2"/>
-      <c r="P117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q117" s="2"/>
-      <c r="R117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="AG117" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH117" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI117" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ117" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="AK117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM117" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="AN117" t="s" s="2">
-        <v>665</v>
-      </c>
-      <c r="AO117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP117" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="118" hidden="true">
-      <c r="A118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="B118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="C118" s="2"/>
-      <c r="D118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E118" s="2"/>
-      <c r="F118" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G118" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J118" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K118" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="L118" t="s" s="2">
-        <v>668</v>
-      </c>
-      <c r="M118" t="s" s="2">
-        <v>669</v>
-      </c>
-      <c r="N118" t="s" s="2">
-        <v>670</v>
-      </c>
-      <c r="O118" s="2"/>
-      <c r="P118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q118" s="2"/>
-      <c r="R118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="AG118" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH118" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI118" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ118" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="AK118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM118" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="AN118" t="s" s="2">
-        <v>671</v>
-      </c>
-      <c r="AO118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP118" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="119" hidden="true">
-      <c r="A119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="B119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="C119" s="2"/>
-      <c r="D119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E119" s="2"/>
-      <c r="F119" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G119" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H119" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J119" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K119" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="L119" t="s" s="2">
-        <v>673</v>
-      </c>
-      <c r="M119" t="s" s="2">
-        <v>673</v>
-      </c>
-      <c r="N119" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="O119" t="s" s="2">
-        <v>675</v>
-      </c>
-      <c r="P119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q119" s="2"/>
-      <c r="R119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="AG119" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH119" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI119" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ119" t="s" s="2">
-        <v>676</v>
-      </c>
-      <c r="AK119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM119" t="s" s="2">
-        <v>677</v>
-      </c>
-      <c r="AN119" t="s" s="2">
-        <v>678</v>
-      </c>
-      <c r="AO119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP119" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="120" hidden="true">
-      <c r="A120" t="s" s="2">
-        <v>679</v>
-      </c>
-      <c r="B120" t="s" s="2">
-        <v>679</v>
-      </c>
-      <c r="C120" s="2"/>
-      <c r="D120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E120" s="2"/>
-      <c r="F120" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G120" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K120" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="L120" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N120" s="2"/>
-      <c r="O120" s="2"/>
-      <c r="P120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q120" s="2"/>
-      <c r="R120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF120" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="AG120" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH120" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN120" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="AO120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP120" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="121" hidden="true">
-      <c r="A121" t="s" s="2">
-        <v>680</v>
-      </c>
-      <c r="B121" t="s" s="2">
-        <v>680</v>
-      </c>
-      <c r="C121" s="2"/>
-      <c r="D121" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="E121" s="2"/>
-      <c r="F121" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G121" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K121" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="L121" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="M121" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N121" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O121" s="2"/>
-      <c r="P121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q121" s="2"/>
-      <c r="R121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB121" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AC121" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="AD121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE121" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="AF121" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="AG121" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH121" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI121" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ121" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="AK121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN121" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AO121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP121" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="122" hidden="true">
-      <c r="A122" t="s" s="2">
-        <v>681</v>
-      </c>
-      <c r="B122" t="s" s="2">
-        <v>681</v>
-      </c>
-      <c r="C122" s="2"/>
-      <c r="D122" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="E122" s="2"/>
-      <c r="F122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G122" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I122" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="J122" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K122" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="L122" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>615</v>
-      </c>
-      <c r="N122" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O122" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="P122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q122" s="2"/>
-      <c r="R122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF122" t="s" s="2">
-        <v>616</v>
-      </c>
-      <c r="AG122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH122" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI122" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ122" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="AK122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN122" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AO122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP122" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="123" hidden="true">
-      <c r="A123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="B123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="C123" s="2"/>
-      <c r="D123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E123" s="2"/>
-      <c r="F123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="G123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H123" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J123" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K123" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L123" t="s" s="2">
-        <v>683</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>684</v>
-      </c>
-      <c r="N123" t="s" s="2">
-        <v>685</v>
-      </c>
-      <c r="O123" t="s" s="2">
-        <v>686</v>
-      </c>
-      <c r="P123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q123" s="2"/>
-      <c r="R123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X123" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y123" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="Z123" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="AA123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="AG123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AH123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI123" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ123" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL123" t="s" s="2">
-        <v>687</v>
-      </c>
-      <c r="AM123" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="AN123" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="AO123" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="AP123" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="124" hidden="true">
-      <c r="A124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="B124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="C124" s="2"/>
-      <c r="D124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E124" s="2"/>
-      <c r="F124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G124" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H124" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J124" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K124" t="s" s="2">
-        <v>689</v>
-      </c>
-      <c r="L124" t="s" s="2">
-        <v>690</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>691</v>
-      </c>
-      <c r="N124" t="s" s="2">
-        <v>692</v>
-      </c>
-      <c r="O124" t="s" s="2">
-        <v>442</v>
-      </c>
-      <c r="P124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q124" s="2"/>
-      <c r="R124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X124" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="Y124" t="s" s="2">
-        <v>693</v>
-      </c>
-      <c r="Z124" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="AA124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="AG124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH124" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI124" t="s" s="2">
-        <v>695</v>
-      </c>
-      <c r="AJ124" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL124" t="s" s="2">
-        <v>696</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="AN124" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="AO124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP124" t="s" s="2">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="125" hidden="true">
-      <c r="A125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="B125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="C125" s="2"/>
-      <c r="D125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E125" s="2"/>
-      <c r="F125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G125" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H125" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K125" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L125" t="s" s="2">
-        <v>698</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>699</v>
-      </c>
-      <c r="N125" t="s" s="2">
-        <v>700</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>509</v>
-      </c>
-      <c r="P125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q125" s="2"/>
-      <c r="R125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X125" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y125" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="Z125" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="AA125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="AG125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH125" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI125" t="s" s="2">
-        <v>701</v>
-      </c>
-      <c r="AJ125" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AN125" t="s" s="2">
-        <v>513</v>
-      </c>
-      <c r="AO125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP125" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="126" hidden="true">
-      <c r="A126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="B126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="C126" s="2"/>
-      <c r="D126" t="s" s="2">
-        <v>526</v>
-      </c>
-      <c r="E126" s="2"/>
-      <c r="F126" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G126" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K126" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L126" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>528</v>
-      </c>
-      <c r="N126" t="s" s="2">
-        <v>529</v>
-      </c>
-      <c r="O126" t="s" s="2">
-        <v>530</v>
-      </c>
-      <c r="P126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q126" s="2"/>
-      <c r="R126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X126" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y126" t="s" s="2">
-        <v>703</v>
-      </c>
-      <c r="Z126" t="s" s="2">
-        <v>531</v>
-      </c>
-      <c r="AA126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="AG126" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH126" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI126" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ126" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL126" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="AM126" t="s" s="2">
-        <v>533</v>
-      </c>
-      <c r="AN126" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="AO126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP126" t="s" s="2">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="127" hidden="true">
-      <c r="A127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="B127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="C127" s="2"/>
-      <c r="D127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E127" s="2"/>
-      <c r="F127" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G127" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K127" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="L127" t="s" s="2">
-        <v>705</v>
-      </c>
-      <c r="M127" t="s" s="2">
-        <v>706</v>
-      </c>
-      <c r="N127" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O127" t="s" s="2">
-        <v>606</v>
-      </c>
-      <c r="P127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q127" s="2"/>
-      <c r="R127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="AG127" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH127" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM127" t="s" s="2">
-        <v>608</v>
-      </c>
-      <c r="AN127" t="s" s="2">
-        <v>609</v>
-      </c>
-      <c r="AO127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP127" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP127">
+  <autoFilter ref="A1:AP116">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -17940,7 +16577,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI126">
+  <conditionalFormatting sqref="A2:AI115">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Ajout du profil saturation en oxygène (#80)
* add oxygen sat profile

* correct value slicing error

* uniformise meta.source

* add J147 Method Heartrate binding to sat method d94b4fdafe41265c49d201b484b36dabfe0155a0
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
+++ b/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$127</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4491" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4914" uniqueCount="707">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-28T12:15:35+00:00</t>
+    <t>2023-11-28T12:22:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1792,6 +1792,39 @@
   </si>
   <si>
     <t>methodCode</t>
+  </si>
+  <si>
+    <t>Observation.method.id</t>
+  </si>
+  <si>
+    <t>Observation.method.extension</t>
+  </si>
+  <si>
+    <t>Observation.method.coding</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.id</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.extension</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.system</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.version</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.code</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.display</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.userSelected</t>
+  </si>
+  <si>
+    <t>Observation.method.text</t>
   </si>
   <si>
     <t>Observation.specimen</t>
@@ -2504,7 +2537,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP116"/>
+  <dimension ref="A1:AP127"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.58984375" customWidth="true" bestFit="true"/>
@@ -2531,7 +2564,7 @@
     <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="109.11328125" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="111.65625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
@@ -13685,7 +13718,7 @@
         <v>91</v>
       </c>
       <c r="H93" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I93" t="s" s="2">
         <v>80</v>
@@ -13731,9 +13764,11 @@
         <v>80</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y93" s="2"/>
+        <v>251</v>
+      </c>
+      <c r="Y93" t="s" s="2">
+        <v>569</v>
+      </c>
       <c r="Z93" t="s" s="2">
         <v>569</v>
       </c>
@@ -13814,17 +13849,15 @@
         <v>80</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>573</v>
+        <v>107</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>574</v>
+        <v>108</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>575</v>
-      </c>
-      <c r="N94" t="s" s="2">
-        <v>576</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N94" s="2"/>
       <c r="O94" s="2"/>
       <c r="P94" t="s" s="2">
         <v>80</v>
@@ -13873,7 +13906,7 @@
         <v>80</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>572</v>
+        <v>110</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
@@ -13882,47 +13915,47 @@
         <v>91</v>
       </c>
       <c r="AI94" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>233</v>
+        <v>80</v>
       </c>
       <c r="AK94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL94" t="s" s="2">
-        <v>577</v>
+        <v>80</v>
       </c>
       <c r="AM94" t="s" s="2">
-        <v>578</v>
+        <v>80</v>
       </c>
       <c r="AN94" t="s" s="2">
-        <v>579</v>
+        <v>111</v>
       </c>
       <c r="AO94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP94" t="s" s="2">
-        <v>580</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>581</v>
+        <v>573</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>581</v>
+        <v>573</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E95" s="2"/>
       <c r="F95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H95" t="s" s="2">
         <v>80</v>
@@ -13934,16 +13967,16 @@
         <v>80</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>582</v>
+        <v>114</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>583</v>
+        <v>115</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>584</v>
+        <v>116</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>585</v>
+        <v>117</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -13981,57 +14014,57 @@
         <v>80</v>
       </c>
       <c r="AB95" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC95" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE95" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>581</v>
+        <v>121</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH95" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI95" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>233</v>
+        <v>122</v>
       </c>
       <c r="AK95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>586</v>
+        <v>80</v>
       </c>
       <c r="AM95" t="s" s="2">
-        <v>587</v>
+        <v>80</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>588</v>
+        <v>105</v>
       </c>
       <c r="AO95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP95" t="s" s="2">
-        <v>589</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>590</v>
+        <v>574</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>590</v>
+        <v>574</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -14051,22 +14084,22 @@
         <v>80</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K96" t="s" s="2">
-        <v>591</v>
+        <v>147</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>592</v>
+        <v>279</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>593</v>
+        <v>280</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>594</v>
+        <v>281</v>
       </c>
       <c r="O96" t="s" s="2">
-        <v>595</v>
+        <v>282</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>80</v>
@@ -14115,7 +14148,7 @@
         <v>80</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>590</v>
+        <v>283</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>78</v>
@@ -14127,7 +14160,7 @@
         <v>103</v>
       </c>
       <c r="AJ96" t="s" s="2">
-        <v>596</v>
+        <v>104</v>
       </c>
       <c r="AK96" t="s" s="2">
         <v>80</v>
@@ -14136,10 +14169,10 @@
         <v>80</v>
       </c>
       <c r="AM96" t="s" s="2">
-        <v>597</v>
+        <v>284</v>
       </c>
       <c r="AN96" t="s" s="2">
-        <v>598</v>
+        <v>285</v>
       </c>
       <c r="AO96" t="s" s="2">
         <v>80</v>
@@ -14150,10 +14183,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>599</v>
+        <v>575</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>599</v>
+        <v>575</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -14268,10 +14301,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>600</v>
+        <v>576</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>600</v>
+        <v>576</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -14388,45 +14421,45 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>601</v>
+        <v>577</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>601</v>
+        <v>577</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
-        <v>602</v>
+        <v>80</v>
       </c>
       <c r="E99" s="2"/>
       <c r="F99" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H99" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I99" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J99" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>603</v>
+        <v>292</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>604</v>
+        <v>293</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>117</v>
+        <v>294</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>215</v>
+        <v>295</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>80</v>
@@ -14475,19 +14508,19 @@
         <v>80</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>605</v>
+        <v>297</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH99" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI99" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ99" t="s" s="2">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="AK99" t="s" s="2">
         <v>80</v>
@@ -14496,10 +14529,10 @@
         <v>80</v>
       </c>
       <c r="AM99" t="s" s="2">
-        <v>80</v>
+        <v>298</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>105</v>
+        <v>299</v>
       </c>
       <c r="AO99" t="s" s="2">
         <v>80</v>
@@ -14510,10 +14543,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>606</v>
+        <v>578</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>606</v>
+        <v>578</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -14533,19 +14566,19 @@
         <v>80</v>
       </c>
       <c r="J100" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>607</v>
+        <v>107</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>608</v>
+        <v>302</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>609</v>
+        <v>303</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>610</v>
+        <v>304</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -14595,7 +14628,7 @@
         <v>80</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>606</v>
+        <v>305</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>78</v>
@@ -14604,10 +14637,10 @@
         <v>91</v>
       </c>
       <c r="AI100" t="s" s="2">
-        <v>611</v>
+        <v>103</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>612</v>
+        <v>104</v>
       </c>
       <c r="AK100" t="s" s="2">
         <v>80</v>
@@ -14616,10 +14649,10 @@
         <v>80</v>
       </c>
       <c r="AM100" t="s" s="2">
-        <v>613</v>
+        <v>306</v>
       </c>
       <c r="AN100" t="s" s="2">
-        <v>614</v>
+        <v>307</v>
       </c>
       <c r="AO100" t="s" s="2">
         <v>80</v>
@@ -14630,10 +14663,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>615</v>
+        <v>579</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>615</v>
+        <v>579</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14641,7 +14674,7 @@
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G101" t="s" s="2">
         <v>91</v>
@@ -14653,21 +14686,23 @@
         <v>80</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>607</v>
+        <v>171</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>616</v>
+        <v>310</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>617</v>
+        <v>311</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>610</v>
-      </c>
-      <c r="O101" s="2"/>
+        <v>312</v>
+      </c>
+      <c r="O101" t="s" s="2">
+        <v>313</v>
+      </c>
       <c r="P101" t="s" s="2">
         <v>80</v>
       </c>
@@ -14715,7 +14750,7 @@
         <v>80</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>615</v>
+        <v>315</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>78</v>
@@ -14724,10 +14759,10 @@
         <v>91</v>
       </c>
       <c r="AI101" t="s" s="2">
-        <v>611</v>
+        <v>103</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>612</v>
+        <v>104</v>
       </c>
       <c r="AK101" t="s" s="2">
         <v>80</v>
@@ -14736,10 +14771,10 @@
         <v>80</v>
       </c>
       <c r="AM101" t="s" s="2">
-        <v>613</v>
+        <v>316</v>
       </c>
       <c r="AN101" t="s" s="2">
-        <v>618</v>
+        <v>317</v>
       </c>
       <c r="AO101" t="s" s="2">
         <v>80</v>
@@ -14750,10 +14785,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>619</v>
+        <v>580</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>619</v>
+        <v>580</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14773,22 +14808,22 @@
         <v>80</v>
       </c>
       <c r="J102" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>260</v>
+        <v>107</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>620</v>
+        <v>320</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>621</v>
+        <v>321</v>
       </c>
       <c r="N102" t="s" s="2">
-        <v>622</v>
+        <v>312</v>
       </c>
       <c r="O102" t="s" s="2">
-        <v>623</v>
+        <v>322</v>
       </c>
       <c r="P102" t="s" s="2">
         <v>80</v>
@@ -14813,13 +14848,13 @@
         <v>80</v>
       </c>
       <c r="X102" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="Y102" t="s" s="2">
-        <v>624</v>
+        <v>80</v>
       </c>
       <c r="Z102" t="s" s="2">
-        <v>625</v>
+        <v>80</v>
       </c>
       <c r="AA102" t="s" s="2">
         <v>80</v>
@@ -14837,7 +14872,7 @@
         <v>80</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>619</v>
+        <v>323</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>78</v>
@@ -14855,13 +14890,13 @@
         <v>80</v>
       </c>
       <c r="AL102" t="s" s="2">
-        <v>626</v>
+        <v>80</v>
       </c>
       <c r="AM102" t="s" s="2">
-        <v>627</v>
+        <v>324</v>
       </c>
       <c r="AN102" t="s" s="2">
-        <v>534</v>
+        <v>325</v>
       </c>
       <c r="AO102" t="s" s="2">
         <v>80</v>
@@ -14872,10 +14907,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>628</v>
+        <v>581</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>628</v>
+        <v>581</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14886,7 +14921,7 @@
         <v>78</v>
       </c>
       <c r="G103" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H103" t="s" s="2">
         <v>80</v>
@@ -14895,22 +14930,22 @@
         <v>80</v>
       </c>
       <c r="J103" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>260</v>
+        <v>328</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>629</v>
+        <v>329</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>630</v>
+        <v>330</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>631</v>
+        <v>331</v>
       </c>
       <c r="O103" t="s" s="2">
-        <v>632</v>
+        <v>332</v>
       </c>
       <c r="P103" t="s" s="2">
         <v>80</v>
@@ -14935,13 +14970,13 @@
         <v>80</v>
       </c>
       <c r="X103" t="s" s="2">
-        <v>161</v>
+        <v>80</v>
       </c>
       <c r="Y103" t="s" s="2">
-        <v>633</v>
+        <v>80</v>
       </c>
       <c r="Z103" t="s" s="2">
-        <v>634</v>
+        <v>80</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>80</v>
@@ -14959,13 +14994,13 @@
         <v>80</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>628</v>
+        <v>333</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH103" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI103" t="s" s="2">
         <v>103</v>
@@ -14977,13 +15012,13 @@
         <v>80</v>
       </c>
       <c r="AL103" t="s" s="2">
-        <v>626</v>
+        <v>80</v>
       </c>
       <c r="AM103" t="s" s="2">
-        <v>627</v>
+        <v>334</v>
       </c>
       <c r="AN103" t="s" s="2">
-        <v>534</v>
+        <v>335</v>
       </c>
       <c r="AO103" t="s" s="2">
         <v>80</v>
@@ -14994,10 +15029,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>635</v>
+        <v>582</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>635</v>
+        <v>582</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -15017,22 +15052,22 @@
         <v>80</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K104" t="s" s="2">
-        <v>636</v>
+        <v>107</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>637</v>
+        <v>338</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>638</v>
+        <v>339</v>
       </c>
       <c r="N104" t="s" s="2">
-        <v>639</v>
+        <v>340</v>
       </c>
       <c r="O104" t="s" s="2">
-        <v>640</v>
+        <v>341</v>
       </c>
       <c r="P104" t="s" s="2">
         <v>80</v>
@@ -15081,7 +15116,7 @@
         <v>80</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>635</v>
+        <v>342</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>78</v>
@@ -15093,7 +15128,7 @@
         <v>103</v>
       </c>
       <c r="AJ104" t="s" s="2">
-        <v>641</v>
+        <v>104</v>
       </c>
       <c r="AK104" t="s" s="2">
         <v>80</v>
@@ -15102,10 +15137,10 @@
         <v>80</v>
       </c>
       <c r="AM104" t="s" s="2">
-        <v>642</v>
+        <v>343</v>
       </c>
       <c r="AN104" t="s" s="2">
-        <v>643</v>
+        <v>344</v>
       </c>
       <c r="AO104" t="s" s="2">
         <v>80</v>
@@ -15116,10 +15151,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>644</v>
+        <v>583</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>644</v>
+        <v>583</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -15142,16 +15177,16 @@
         <v>80</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>107</v>
+        <v>584</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>645</v>
+        <v>585</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>646</v>
+        <v>586</v>
       </c>
       <c r="N105" t="s" s="2">
-        <v>312</v>
+        <v>587</v>
       </c>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
@@ -15201,7 +15236,7 @@
         <v>80</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>644</v>
+        <v>583</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>78</v>
@@ -15213,33 +15248,33 @@
         <v>103</v>
       </c>
       <c r="AJ105" t="s" s="2">
-        <v>104</v>
+        <v>233</v>
       </c>
       <c r="AK105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL105" t="s" s="2">
-        <v>80</v>
+        <v>588</v>
       </c>
       <c r="AM105" t="s" s="2">
-        <v>613</v>
+        <v>589</v>
       </c>
       <c r="AN105" t="s" s="2">
-        <v>647</v>
+        <v>590</v>
       </c>
       <c r="AO105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP105" t="s" s="2">
-        <v>80</v>
+        <v>591</v>
       </c>
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>648</v>
+        <v>592</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>648</v>
+        <v>592</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -15250,7 +15285,7 @@
         <v>78</v>
       </c>
       <c r="G106" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H106" t="s" s="2">
         <v>80</v>
@@ -15259,19 +15294,19 @@
         <v>80</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K106" t="s" s="2">
-        <v>649</v>
+        <v>593</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>650</v>
+        <v>594</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>651</v>
+        <v>595</v>
       </c>
       <c r="N106" t="s" s="2">
-        <v>652</v>
+        <v>596</v>
       </c>
       <c r="O106" s="2"/>
       <c r="P106" t="s" s="2">
@@ -15321,13 +15356,13 @@
         <v>80</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>648</v>
+        <v>592</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH106" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI106" t="s" s="2">
         <v>103</v>
@@ -15339,27 +15374,27 @@
         <v>80</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>80</v>
+        <v>597</v>
       </c>
       <c r="AM106" t="s" s="2">
-        <v>653</v>
+        <v>598</v>
       </c>
       <c r="AN106" t="s" s="2">
-        <v>654</v>
+        <v>599</v>
       </c>
       <c r="AO106" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP106" t="s" s="2">
-        <v>80</v>
+        <v>600</v>
       </c>
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>655</v>
+        <v>601</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>655</v>
+        <v>601</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -15379,21 +15414,23 @@
         <v>80</v>
       </c>
       <c r="J107" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>656</v>
+        <v>602</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>657</v>
+        <v>603</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>658</v>
+        <v>604</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="O107" s="2"/>
+        <v>605</v>
+      </c>
+      <c r="O107" t="s" s="2">
+        <v>606</v>
+      </c>
       <c r="P107" t="s" s="2">
         <v>80</v>
       </c>
@@ -15441,7 +15478,7 @@
         <v>80</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>655</v>
+        <v>601</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>78</v>
@@ -15453,7 +15490,7 @@
         <v>103</v>
       </c>
       <c r="AJ107" t="s" s="2">
-        <v>233</v>
+        <v>607</v>
       </c>
       <c r="AK107" t="s" s="2">
         <v>80</v>
@@ -15462,10 +15499,10 @@
         <v>80</v>
       </c>
       <c r="AM107" t="s" s="2">
-        <v>653</v>
+        <v>608</v>
       </c>
       <c r="AN107" t="s" s="2">
-        <v>660</v>
+        <v>609</v>
       </c>
       <c r="AO107" t="s" s="2">
         <v>80</v>
@@ -15476,10 +15513,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>661</v>
+        <v>610</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>661</v>
+        <v>610</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -15490,32 +15527,28 @@
         <v>78</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H108" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I108" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J108" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>591</v>
+        <v>107</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>662</v>
+        <v>108</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>662</v>
-      </c>
-      <c r="N108" t="s" s="2">
-        <v>663</v>
-      </c>
-      <c r="O108" t="s" s="2">
-        <v>664</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N108" s="2"/>
+      <c r="O108" s="2"/>
       <c r="P108" t="s" s="2">
         <v>80</v>
       </c>
@@ -15563,19 +15596,19 @@
         <v>80</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>661</v>
+        <v>110</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH108" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI108" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ108" t="s" s="2">
-        <v>665</v>
+        <v>80</v>
       </c>
       <c r="AK108" t="s" s="2">
         <v>80</v>
@@ -15584,10 +15617,10 @@
         <v>80</v>
       </c>
       <c r="AM108" t="s" s="2">
-        <v>666</v>
+        <v>80</v>
       </c>
       <c r="AN108" t="s" s="2">
-        <v>667</v>
+        <v>111</v>
       </c>
       <c r="AO108" t="s" s="2">
         <v>80</v>
@@ -15598,21 +15631,21 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>668</v>
+        <v>611</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>668</v>
+        <v>611</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E109" s="2"/>
       <c r="F109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H109" t="s" s="2">
         <v>80</v>
@@ -15624,15 +15657,17 @@
         <v>80</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N109" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="N109" t="s" s="2">
+        <v>117</v>
+      </c>
       <c r="O109" s="2"/>
       <c r="P109" t="s" s="2">
         <v>80</v>
@@ -15669,31 +15704,31 @@
         <v>80</v>
       </c>
       <c r="AB109" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC109" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD109" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE109" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH109" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI109" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ109" t="s" s="2">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="AK109" t="s" s="2">
         <v>80</v>
@@ -15705,7 +15740,7 @@
         <v>80</v>
       </c>
       <c r="AN109" t="s" s="2">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="AO109" t="s" s="2">
         <v>80</v>
@@ -15716,14 +15751,14 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>669</v>
+        <v>612</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>669</v>
+        <v>612</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
-        <v>113</v>
+        <v>613</v>
       </c>
       <c r="E110" s="2"/>
       <c r="F110" t="s" s="2">
@@ -15736,24 +15771,26 @@
         <v>80</v>
       </c>
       <c r="I110" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J110" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K110" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>115</v>
+        <v>614</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>116</v>
+        <v>615</v>
       </c>
       <c r="N110" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O110" s="2"/>
+      <c r="O110" t="s" s="2">
+        <v>215</v>
+      </c>
       <c r="P110" t="s" s="2">
         <v>80</v>
       </c>
@@ -15789,19 +15826,19 @@
         <v>80</v>
       </c>
       <c r="AB110" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC110" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE110" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>121</v>
+        <v>616</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>78</v>
@@ -15836,46 +15873,44 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>670</v>
+        <v>617</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>670</v>
+        <v>617</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
-        <v>602</v>
+        <v>80</v>
       </c>
       <c r="E111" s="2"/>
       <c r="F111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G111" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H111" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I111" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J111" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>114</v>
+        <v>618</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>603</v>
+        <v>619</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>604</v>
+        <v>620</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O111" t="s" s="2">
-        <v>215</v>
-      </c>
+        <v>621</v>
+      </c>
+      <c r="O111" s="2"/>
       <c r="P111" t="s" s="2">
         <v>80</v>
       </c>
@@ -15923,19 +15958,19 @@
         <v>80</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>605</v>
+        <v>617</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH111" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI111" t="s" s="2">
-        <v>103</v>
+        <v>622</v>
       </c>
       <c r="AJ111" t="s" s="2">
-        <v>122</v>
+        <v>623</v>
       </c>
       <c r="AK111" t="s" s="2">
         <v>80</v>
@@ -15944,10 +15979,10 @@
         <v>80</v>
       </c>
       <c r="AM111" t="s" s="2">
-        <v>80</v>
+        <v>624</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>105</v>
+        <v>625</v>
       </c>
       <c r="AO111" t="s" s="2">
         <v>80</v>
@@ -15958,10 +15993,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>671</v>
+        <v>626</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>671</v>
+        <v>626</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -15969,35 +16004,33 @@
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H112" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J112" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>260</v>
+        <v>618</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>672</v>
+        <v>627</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>673</v>
+        <v>628</v>
       </c>
       <c r="N112" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="O112" t="s" s="2">
-        <v>675</v>
-      </c>
+        <v>621</v>
+      </c>
+      <c r="O112" s="2"/>
       <c r="P112" t="s" s="2">
         <v>80</v>
       </c>
@@ -16021,13 +16054,13 @@
         <v>80</v>
       </c>
       <c r="X112" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="Y112" t="s" s="2">
-        <v>351</v>
+        <v>80</v>
       </c>
       <c r="Z112" t="s" s="2">
-        <v>352</v>
+        <v>80</v>
       </c>
       <c r="AA112" t="s" s="2">
         <v>80</v>
@@ -16045,34 +16078,34 @@
         <v>80</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>671</v>
+        <v>626</v>
       </c>
       <c r="AG112" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="AH112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="AI112" t="s" s="2">
-        <v>103</v>
+        <v>622</v>
       </c>
       <c r="AJ112" t="s" s="2">
-        <v>104</v>
+        <v>623</v>
       </c>
       <c r="AK112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>676</v>
+        <v>80</v>
       </c>
       <c r="AM112" t="s" s="2">
-        <v>355</v>
+        <v>624</v>
       </c>
       <c r="AN112" t="s" s="2">
-        <v>356</v>
+        <v>629</v>
       </c>
       <c r="AO112" t="s" s="2">
-        <v>357</v>
+        <v>80</v>
       </c>
       <c r="AP112" t="s" s="2">
         <v>80</v>
@@ -16080,10 +16113,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>677</v>
+        <v>630</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>677</v>
+        <v>630</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -16097,28 +16130,28 @@
         <v>91</v>
       </c>
       <c r="H113" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J113" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>678</v>
+        <v>260</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>679</v>
+        <v>631</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>680</v>
+        <v>632</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>681</v>
+        <v>633</v>
       </c>
       <c r="O113" t="s" s="2">
-        <v>442</v>
+        <v>634</v>
       </c>
       <c r="P113" t="s" s="2">
         <v>80</v>
@@ -16143,13 +16176,13 @@
         <v>80</v>
       </c>
       <c r="X113" t="s" s="2">
-        <v>251</v>
+        <v>175</v>
       </c>
       <c r="Y113" t="s" s="2">
-        <v>682</v>
+        <v>635</v>
       </c>
       <c r="Z113" t="s" s="2">
-        <v>683</v>
+        <v>636</v>
       </c>
       <c r="AA113" t="s" s="2">
         <v>80</v>
@@ -16167,7 +16200,7 @@
         <v>80</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>677</v>
+        <v>630</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
@@ -16176,7 +16209,7 @@
         <v>91</v>
       </c>
       <c r="AI113" t="s" s="2">
-        <v>684</v>
+        <v>103</v>
       </c>
       <c r="AJ113" t="s" s="2">
         <v>104</v>
@@ -16185,27 +16218,27 @@
         <v>80</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>685</v>
+        <v>637</v>
       </c>
       <c r="AM113" t="s" s="2">
-        <v>447</v>
+        <v>638</v>
       </c>
       <c r="AN113" t="s" s="2">
-        <v>448</v>
+        <v>534</v>
       </c>
       <c r="AO113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP113" t="s" s="2">
-        <v>449</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -16216,10 +16249,10 @@
         <v>78</v>
       </c>
       <c r="G114" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H114" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I114" t="s" s="2">
         <v>80</v>
@@ -16231,16 +16264,16 @@
         <v>260</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>687</v>
+        <v>640</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>688</v>
+        <v>641</v>
       </c>
       <c r="N114" t="s" s="2">
-        <v>689</v>
+        <v>642</v>
       </c>
       <c r="O114" t="s" s="2">
-        <v>509</v>
+        <v>643</v>
       </c>
       <c r="P114" t="s" s="2">
         <v>80</v>
@@ -16265,13 +16298,13 @@
         <v>80</v>
       </c>
       <c r="X114" t="s" s="2">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="Y114" t="s" s="2">
-        <v>510</v>
+        <v>644</v>
       </c>
       <c r="Z114" t="s" s="2">
-        <v>511</v>
+        <v>645</v>
       </c>
       <c r="AA114" t="s" s="2">
         <v>80</v>
@@ -16289,16 +16322,16 @@
         <v>80</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH114" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI114" t="s" s="2">
-        <v>690</v>
+        <v>103</v>
       </c>
       <c r="AJ114" t="s" s="2">
         <v>104</v>
@@ -16307,13 +16340,13 @@
         <v>80</v>
       </c>
       <c r="AL114" t="s" s="2">
-        <v>80</v>
+        <v>637</v>
       </c>
       <c r="AM114" t="s" s="2">
-        <v>105</v>
+        <v>638</v>
       </c>
       <c r="AN114" t="s" s="2">
-        <v>513</v>
+        <v>534</v>
       </c>
       <c r="AO114" t="s" s="2">
         <v>80</v>
@@ -16324,21 +16357,21 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
-        <v>526</v>
+        <v>80</v>
       </c>
       <c r="E115" s="2"/>
       <c r="F115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G115" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H115" t="s" s="2">
         <v>80</v>
@@ -16350,19 +16383,19 @@
         <v>80</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>260</v>
+        <v>647</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>527</v>
+        <v>648</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>528</v>
+        <v>649</v>
       </c>
       <c r="N115" t="s" s="2">
-        <v>529</v>
+        <v>650</v>
       </c>
       <c r="O115" t="s" s="2">
-        <v>530</v>
+        <v>651</v>
       </c>
       <c r="P115" t="s" s="2">
         <v>80</v>
@@ -16387,13 +16420,13 @@
         <v>80</v>
       </c>
       <c r="X115" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="Y115" t="s" s="2">
-        <v>692</v>
+        <v>80</v>
       </c>
       <c r="Z115" t="s" s="2">
-        <v>531</v>
+        <v>80</v>
       </c>
       <c r="AA115" t="s" s="2">
         <v>80</v>
@@ -16411,45 +16444,45 @@
         <v>80</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH115" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI115" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ115" t="s" s="2">
-        <v>104</v>
+        <v>652</v>
       </c>
       <c r="AK115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>532</v>
+        <v>80</v>
       </c>
       <c r="AM115" t="s" s="2">
-        <v>533</v>
+        <v>653</v>
       </c>
       <c r="AN115" t="s" s="2">
-        <v>534</v>
+        <v>654</v>
       </c>
       <c r="AO115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP115" t="s" s="2">
-        <v>535</v>
+        <v>80</v>
       </c>
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>693</v>
+        <v>655</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>693</v>
+        <v>655</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -16460,7 +16493,7 @@
         <v>78</v>
       </c>
       <c r="G116" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H116" t="s" s="2">
         <v>80</v>
@@ -16472,20 +16505,18 @@
         <v>80</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>694</v>
+        <v>656</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>695</v>
+        <v>657</v>
       </c>
       <c r="N116" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="O116" t="s" s="2">
-        <v>595</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="O116" s="2"/>
       <c r="P116" t="s" s="2">
         <v>80</v>
       </c>
@@ -16533,41 +16564,1373 @@
         <v>80</v>
       </c>
       <c r="AF116" t="s" s="2">
+        <v>655</v>
+      </c>
+      <c r="AG116" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH116" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI116" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ116" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK116" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL116" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM116" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="AN116" t="s" s="2">
+        <v>658</v>
+      </c>
+      <c r="AO116" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP116" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="117" hidden="true">
+      <c r="A117" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="B117" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="C117" s="2"/>
+      <c r="D117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E117" s="2"/>
+      <c r="F117" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G117" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J117" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K117" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="L117" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="M117" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="N117" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="O117" s="2"/>
+      <c r="P117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q117" s="2"/>
+      <c r="R117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF117" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="AG117" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH117" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI117" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ117" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="AK117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM117" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="AN117" t="s" s="2">
+        <v>665</v>
+      </c>
+      <c r="AO117" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP117" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="118" hidden="true">
+      <c r="A118" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="B118" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="C118" s="2"/>
+      <c r="D118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E118" s="2"/>
+      <c r="F118" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G118" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J118" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K118" t="s" s="2">
+        <v>667</v>
+      </c>
+      <c r="L118" t="s" s="2">
+        <v>668</v>
+      </c>
+      <c r="M118" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="N118" t="s" s="2">
+        <v>670</v>
+      </c>
+      <c r="O118" s="2"/>
+      <c r="P118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q118" s="2"/>
+      <c r="R118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF118" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="AG118" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH118" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI118" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ118" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="AK118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM118" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="AN118" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="AO118" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP118" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="119" hidden="true">
+      <c r="A119" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="B119" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="C119" s="2"/>
+      <c r="D119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E119" s="2"/>
+      <c r="F119" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G119" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H119" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J119" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K119" t="s" s="2">
+        <v>602</v>
+      </c>
+      <c r="L119" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="M119" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="N119" t="s" s="2">
+        <v>674</v>
+      </c>
+      <c r="O119" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="P119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q119" s="2"/>
+      <c r="R119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF119" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="AG119" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH119" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI119" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ119" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="AK119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM119" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="AN119" t="s" s="2">
+        <v>678</v>
+      </c>
+      <c r="AO119" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP119" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="120" hidden="true">
+      <c r="A120" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="B120" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="C120" s="2"/>
+      <c r="D120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E120" s="2"/>
+      <c r="F120" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G120" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K120" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="L120" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="M120" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="N120" s="2"/>
+      <c r="O120" s="2"/>
+      <c r="P120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q120" s="2"/>
+      <c r="R120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF120" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="AG120" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH120" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN120" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AO120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP120" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="121" hidden="true">
+      <c r="A121" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="B121" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="C121" s="2"/>
+      <c r="D121" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="E121" s="2"/>
+      <c r="F121" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G121" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K121" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="L121" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="M121" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="N121" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O121" s="2"/>
+      <c r="P121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q121" s="2"/>
+      <c r="R121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB121" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AC121" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AD121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE121" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AF121" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AG121" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH121" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI121" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ121" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN121" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AO121" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP121" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="122" hidden="true">
+      <c r="A122" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="B122" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="C122" s="2"/>
+      <c r="D122" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="E122" s="2"/>
+      <c r="F122" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G122" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I122" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="J122" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K122" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="L122" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="M122" t="s" s="2">
+        <v>615</v>
+      </c>
+      <c r="N122" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O122" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="P122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q122" s="2"/>
+      <c r="R122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF122" t="s" s="2">
+        <v>616</v>
+      </c>
+      <c r="AG122" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH122" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI122" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ122" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN122" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AO122" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP122" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="123" hidden="true">
+      <c r="A123" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="B123" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="C123" s="2"/>
+      <c r="D123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E123" s="2"/>
+      <c r="F123" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="G123" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H123" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J123" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K123" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="L123" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="M123" t="s" s="2">
+        <v>684</v>
+      </c>
+      <c r="N123" t="s" s="2">
+        <v>685</v>
+      </c>
+      <c r="O123" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="P123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q123" s="2"/>
+      <c r="R123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X123" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y123" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="Z123" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="AA123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF123" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="AG123" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AH123" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI123" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ123" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK123" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL123" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="AM123" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AN123" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="AO123" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="AP123" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="124" hidden="true">
+      <c r="A124" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="B124" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="C124" s="2"/>
+      <c r="D124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E124" s="2"/>
+      <c r="F124" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G124" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H124" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J124" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K124" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="L124" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="M124" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="N124" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="O124" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="P124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q124" s="2"/>
+      <c r="R124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X124" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="Y124" t="s" s="2">
         <v>693</v>
       </c>
-      <c r="AG116" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH116" t="s" s="2">
+      <c r="Z124" t="s" s="2">
+        <v>694</v>
+      </c>
+      <c r="AA124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF124" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="AG124" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH124" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI124" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="AJ124" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL124" t="s" s="2">
+        <v>696</v>
+      </c>
+      <c r="AM124" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="AN124" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="AO124" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP124" t="s" s="2">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="125" hidden="true">
+      <c r="A125" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="B125" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="C125" s="2"/>
+      <c r="D125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E125" s="2"/>
+      <c r="F125" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G125" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H125" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K125" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="L125" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="M125" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="N125" t="s" s="2">
+        <v>700</v>
+      </c>
+      <c r="O125" t="s" s="2">
+        <v>509</v>
+      </c>
+      <c r="P125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q125" s="2"/>
+      <c r="R125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X125" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y125" t="s" s="2">
+        <v>510</v>
+      </c>
+      <c r="Z125" t="s" s="2">
+        <v>511</v>
+      </c>
+      <c r="AA125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF125" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="AG125" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH125" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI125" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="AJ125" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM125" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AN125" t="s" s="2">
+        <v>513</v>
+      </c>
+      <c r="AO125" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP125" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="126" hidden="true">
+      <c r="A126" t="s" s="2">
+        <v>702</v>
+      </c>
+      <c r="B126" t="s" s="2">
+        <v>702</v>
+      </c>
+      <c r="C126" s="2"/>
+      <c r="D126" t="s" s="2">
+        <v>526</v>
+      </c>
+      <c r="E126" s="2"/>
+      <c r="F126" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G126" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="AI116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM116" t="s" s="2">
-        <v>597</v>
-      </c>
-      <c r="AN116" t="s" s="2">
-        <v>598</v>
-      </c>
-      <c r="AO116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP116" t="s" s="2">
+      <c r="H126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K126" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="L126" t="s" s="2">
+        <v>527</v>
+      </c>
+      <c r="M126" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="N126" t="s" s="2">
+        <v>529</v>
+      </c>
+      <c r="O126" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="P126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q126" s="2"/>
+      <c r="R126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X126" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y126" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="Z126" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="AA126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF126" t="s" s="2">
+        <v>702</v>
+      </c>
+      <c r="AG126" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH126" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI126" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ126" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL126" t="s" s="2">
+        <v>532</v>
+      </c>
+      <c r="AM126" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="AN126" t="s" s="2">
+        <v>534</v>
+      </c>
+      <c r="AO126" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP126" t="s" s="2">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="127" hidden="true">
+      <c r="A127" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="B127" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="C127" s="2"/>
+      <c r="D127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E127" s="2"/>
+      <c r="F127" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G127" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K127" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="L127" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="M127" t="s" s="2">
+        <v>706</v>
+      </c>
+      <c r="N127" t="s" s="2">
+        <v>605</v>
+      </c>
+      <c r="O127" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="P127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q127" s="2"/>
+      <c r="R127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF127" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="AG127" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH127" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM127" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="AN127" t="s" s="2">
+        <v>609</v>
+      </c>
+      <c r="AO127" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP127" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP116">
+  <autoFilter ref="A1:AP127">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -16577,7 +17940,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI115">
+  <conditionalFormatting sqref="A2:AI126">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Mise à jour page d'accueil et ajout description MDC (#83)
* update index page and md description

* update mdc title 8621218382f501a574f7bb0b4712ae8b7515556a
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
+++ b/ig/main/StructureDefinition-mesures-fr-observation-body-temperature.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$116</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4914" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4491" uniqueCount="696">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-28T12:22:20+00:00</t>
+    <t>2023-11-28T12:44:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1792,39 +1792,6 @@
   </si>
   <si>
     <t>methodCode</t>
-  </si>
-  <si>
-    <t>Observation.method.id</t>
-  </si>
-  <si>
-    <t>Observation.method.extension</t>
-  </si>
-  <si>
-    <t>Observation.method.coding</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.id</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.extension</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.system</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.version</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.code</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.display</t>
-  </si>
-  <si>
-    <t>Observation.method.coding.userSelected</t>
-  </si>
-  <si>
-    <t>Observation.method.text</t>
   </si>
   <si>
     <t>Observation.specimen</t>
@@ -2537,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP127"/>
+  <dimension ref="A1:AP116"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.58984375" customWidth="true" bestFit="true"/>
@@ -2564,7 +2531,7 @@
     <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="109.11328125" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="111.65625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
@@ -13718,7 +13685,7 @@
         <v>91</v>
       </c>
       <c r="H93" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I93" t="s" s="2">
         <v>80</v>
@@ -13764,11 +13731,9 @@
         <v>80</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="Y93" t="s" s="2">
-        <v>569</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="Y93" s="2"/>
       <c r="Z93" t="s" s="2">
         <v>569</v>
       </c>
@@ -13849,15 +13814,17 @@
         <v>80</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>107</v>
+        <v>573</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>108</v>
+        <v>574</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N94" s="2"/>
+        <v>575</v>
+      </c>
+      <c r="N94" t="s" s="2">
+        <v>576</v>
+      </c>
       <c r="O94" s="2"/>
       <c r="P94" t="s" s="2">
         <v>80</v>
@@ -13906,7 +13873,7 @@
         <v>80</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>110</v>
+        <v>572</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
@@ -13915,47 +13882,47 @@
         <v>91</v>
       </c>
       <c r="AI94" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>80</v>
+        <v>233</v>
       </c>
       <c r="AK94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL94" t="s" s="2">
-        <v>80</v>
+        <v>577</v>
       </c>
       <c r="AM94" t="s" s="2">
-        <v>80</v>
+        <v>578</v>
       </c>
       <c r="AN94" t="s" s="2">
-        <v>111</v>
+        <v>579</v>
       </c>
       <c r="AO94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP94" t="s" s="2">
-        <v>80</v>
+        <v>580</v>
       </c>
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E95" s="2"/>
       <c r="F95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H95" t="s" s="2">
         <v>80</v>
@@ -13967,16 +13934,16 @@
         <v>80</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>114</v>
+        <v>582</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>115</v>
+        <v>583</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>116</v>
+        <v>584</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>117</v>
+        <v>585</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -14014,57 +13981,57 @@
         <v>80</v>
       </c>
       <c r="AB95" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC95" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE95" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>121</v>
+        <v>581</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH95" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI95" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>122</v>
+        <v>233</v>
       </c>
       <c r="AK95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>80</v>
+        <v>586</v>
       </c>
       <c r="AM95" t="s" s="2">
-        <v>80</v>
+        <v>587</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>105</v>
+        <v>588</v>
       </c>
       <c r="AO95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP95" t="s" s="2">
-        <v>80</v>
+        <v>589</v>
       </c>
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -14084,22 +14051,22 @@
         <v>80</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K96" t="s" s="2">
-        <v>147</v>
+        <v>591</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>279</v>
+        <v>592</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>280</v>
+        <v>593</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>281</v>
+        <v>594</v>
       </c>
       <c r="O96" t="s" s="2">
-        <v>282</v>
+        <v>595</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>80</v>
@@ -14148,7 +14115,7 @@
         <v>80</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>283</v>
+        <v>590</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>78</v>
@@ -14160,7 +14127,7 @@
         <v>103</v>
       </c>
       <c r="AJ96" t="s" s="2">
-        <v>104</v>
+        <v>596</v>
       </c>
       <c r="AK96" t="s" s="2">
         <v>80</v>
@@ -14169,10 +14136,10 @@
         <v>80</v>
       </c>
       <c r="AM96" t="s" s="2">
-        <v>284</v>
+        <v>597</v>
       </c>
       <c r="AN96" t="s" s="2">
-        <v>285</v>
+        <v>598</v>
       </c>
       <c r="AO96" t="s" s="2">
         <v>80</v>
@@ -14183,10 +14150,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -14301,10 +14268,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>576</v>
+        <v>600</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>576</v>
+        <v>600</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -14421,45 +14388,45 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>577</v>
+        <v>601</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
-        <v>80</v>
+        <v>602</v>
       </c>
       <c r="E99" s="2"/>
       <c r="F99" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H99" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I99" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J99" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>292</v>
+        <v>603</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>293</v>
+        <v>604</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>294</v>
+        <v>117</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>295</v>
+        <v>215</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>80</v>
@@ -14508,19 +14475,19 @@
         <v>80</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>297</v>
+        <v>605</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH99" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI99" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ99" t="s" s="2">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="AK99" t="s" s="2">
         <v>80</v>
@@ -14529,10 +14496,10 @@
         <v>80</v>
       </c>
       <c r="AM99" t="s" s="2">
-        <v>298</v>
+        <v>80</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>299</v>
+        <v>105</v>
       </c>
       <c r="AO99" t="s" s="2">
         <v>80</v>
@@ -14543,10 +14510,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>578</v>
+        <v>606</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>578</v>
+        <v>606</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -14566,19 +14533,19 @@
         <v>80</v>
       </c>
       <c r="J100" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>107</v>
+        <v>607</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>302</v>
+        <v>608</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>303</v>
+        <v>609</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>304</v>
+        <v>610</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -14628,7 +14595,7 @@
         <v>80</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>305</v>
+        <v>606</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>78</v>
@@ -14637,10 +14604,10 @@
         <v>91</v>
       </c>
       <c r="AI100" t="s" s="2">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>104</v>
+        <v>612</v>
       </c>
       <c r="AK100" t="s" s="2">
         <v>80</v>
@@ -14649,10 +14616,10 @@
         <v>80</v>
       </c>
       <c r="AM100" t="s" s="2">
-        <v>306</v>
+        <v>613</v>
       </c>
       <c r="AN100" t="s" s="2">
-        <v>307</v>
+        <v>614</v>
       </c>
       <c r="AO100" t="s" s="2">
         <v>80</v>
@@ -14663,10 +14630,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>579</v>
+        <v>615</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>579</v>
+        <v>615</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14674,7 +14641,7 @@
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G101" t="s" s="2">
         <v>91</v>
@@ -14686,23 +14653,21 @@
         <v>80</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>171</v>
+        <v>607</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>310</v>
+        <v>616</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>311</v>
+        <v>617</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="O101" t="s" s="2">
-        <v>313</v>
-      </c>
+        <v>610</v>
+      </c>
+      <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
         <v>80</v>
       </c>
@@ -14750,7 +14715,7 @@
         <v>80</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>315</v>
+        <v>615</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>78</v>
@@ -14759,10 +14724,10 @@
         <v>91</v>
       </c>
       <c r="AI101" t="s" s="2">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>104</v>
+        <v>612</v>
       </c>
       <c r="AK101" t="s" s="2">
         <v>80</v>
@@ -14771,10 +14736,10 @@
         <v>80</v>
       </c>
       <c r="AM101" t="s" s="2">
-        <v>316</v>
+        <v>613</v>
       </c>
       <c r="AN101" t="s" s="2">
-        <v>317</v>
+        <v>618</v>
       </c>
       <c r="AO101" t="s" s="2">
         <v>80</v>
@@ -14785,10 +14750,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>580</v>
+        <v>619</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>580</v>
+        <v>619</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14808,22 +14773,22 @@
         <v>80</v>
       </c>
       <c r="J102" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>107</v>
+        <v>260</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>320</v>
+        <v>620</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>321</v>
+        <v>621</v>
       </c>
       <c r="N102" t="s" s="2">
-        <v>312</v>
+        <v>622</v>
       </c>
       <c r="O102" t="s" s="2">
-        <v>322</v>
+        <v>623</v>
       </c>
       <c r="P102" t="s" s="2">
         <v>80</v>
@@ -14848,13 +14813,13 @@
         <v>80</v>
       </c>
       <c r="X102" t="s" s="2">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="Y102" t="s" s="2">
-        <v>80</v>
+        <v>624</v>
       </c>
       <c r="Z102" t="s" s="2">
-        <v>80</v>
+        <v>625</v>
       </c>
       <c r="AA102" t="s" s="2">
         <v>80</v>
@@ -14872,7 +14837,7 @@
         <v>80</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>323</v>
+        <v>619</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>78</v>
@@ -14890,13 +14855,13 @@
         <v>80</v>
       </c>
       <c r="AL102" t="s" s="2">
-        <v>80</v>
+        <v>626</v>
       </c>
       <c r="AM102" t="s" s="2">
-        <v>324</v>
+        <v>627</v>
       </c>
       <c r="AN102" t="s" s="2">
-        <v>325</v>
+        <v>534</v>
       </c>
       <c r="AO102" t="s" s="2">
         <v>80</v>
@@ -14907,10 +14872,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>581</v>
+        <v>628</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>581</v>
+        <v>628</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14921,7 +14886,7 @@
         <v>78</v>
       </c>
       <c r="G103" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H103" t="s" s="2">
         <v>80</v>
@@ -14930,22 +14895,22 @@
         <v>80</v>
       </c>
       <c r="J103" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>328</v>
+        <v>260</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>329</v>
+        <v>629</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>330</v>
+        <v>630</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>331</v>
+        <v>631</v>
       </c>
       <c r="O103" t="s" s="2">
-        <v>332</v>
+        <v>632</v>
       </c>
       <c r="P103" t="s" s="2">
         <v>80</v>
@@ -14970,13 +14935,13 @@
         <v>80</v>
       </c>
       <c r="X103" t="s" s="2">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="Y103" t="s" s="2">
-        <v>80</v>
+        <v>633</v>
       </c>
       <c r="Z103" t="s" s="2">
-        <v>80</v>
+        <v>634</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>80</v>
@@ -14994,13 +14959,13 @@
         <v>80</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>333</v>
+        <v>628</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH103" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI103" t="s" s="2">
         <v>103</v>
@@ -15012,13 +14977,13 @@
         <v>80</v>
       </c>
       <c r="AL103" t="s" s="2">
-        <v>80</v>
+        <v>626</v>
       </c>
       <c r="AM103" t="s" s="2">
-        <v>334</v>
+        <v>627</v>
       </c>
       <c r="AN103" t="s" s="2">
-        <v>335</v>
+        <v>534</v>
       </c>
       <c r="AO103" t="s" s="2">
         <v>80</v>
@@ -15029,10 +14994,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>582</v>
+        <v>635</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>582</v>
+        <v>635</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -15052,22 +15017,22 @@
         <v>80</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K104" t="s" s="2">
-        <v>107</v>
+        <v>636</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>338</v>
+        <v>637</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>339</v>
+        <v>638</v>
       </c>
       <c r="N104" t="s" s="2">
-        <v>340</v>
+        <v>639</v>
       </c>
       <c r="O104" t="s" s="2">
-        <v>341</v>
+        <v>640</v>
       </c>
       <c r="P104" t="s" s="2">
         <v>80</v>
@@ -15116,7 +15081,7 @@
         <v>80</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>342</v>
+        <v>635</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>78</v>
@@ -15128,7 +15093,7 @@
         <v>103</v>
       </c>
       <c r="AJ104" t="s" s="2">
-        <v>104</v>
+        <v>641</v>
       </c>
       <c r="AK104" t="s" s="2">
         <v>80</v>
@@ -15137,10 +15102,10 @@
         <v>80</v>
       </c>
       <c r="AM104" t="s" s="2">
-        <v>343</v>
+        <v>642</v>
       </c>
       <c r="AN104" t="s" s="2">
-        <v>344</v>
+        <v>643</v>
       </c>
       <c r="AO104" t="s" s="2">
         <v>80</v>
@@ -15151,10 +15116,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -15177,16 +15142,16 @@
         <v>80</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>584</v>
+        <v>107</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>585</v>
+        <v>645</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>586</v>
+        <v>646</v>
       </c>
       <c r="N105" t="s" s="2">
-        <v>587</v>
+        <v>312</v>
       </c>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
@@ -15236,7 +15201,7 @@
         <v>80</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>583</v>
+        <v>644</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>78</v>
@@ -15248,33 +15213,33 @@
         <v>103</v>
       </c>
       <c r="AJ105" t="s" s="2">
-        <v>233</v>
+        <v>104</v>
       </c>
       <c r="AK105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL105" t="s" s="2">
-        <v>588</v>
+        <v>80</v>
       </c>
       <c r="AM105" t="s" s="2">
-        <v>589</v>
+        <v>613</v>
       </c>
       <c r="AN105" t="s" s="2">
-        <v>590</v>
+        <v>647</v>
       </c>
       <c r="AO105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP105" t="s" s="2">
-        <v>591</v>
+        <v>80</v>
       </c>
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -15285,7 +15250,7 @@
         <v>78</v>
       </c>
       <c r="G106" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H106" t="s" s="2">
         <v>80</v>
@@ -15294,19 +15259,19 @@
         <v>80</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K106" t="s" s="2">
-        <v>593</v>
+        <v>649</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>594</v>
+        <v>650</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>595</v>
+        <v>651</v>
       </c>
       <c r="N106" t="s" s="2">
-        <v>596</v>
+        <v>652</v>
       </c>
       <c r="O106" s="2"/>
       <c r="P106" t="s" s="2">
@@ -15356,13 +15321,13 @@
         <v>80</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>592</v>
+        <v>648</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH106" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI106" t="s" s="2">
         <v>103</v>
@@ -15374,27 +15339,27 @@
         <v>80</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>597</v>
+        <v>80</v>
       </c>
       <c r="AM106" t="s" s="2">
-        <v>598</v>
+        <v>653</v>
       </c>
       <c r="AN106" t="s" s="2">
-        <v>599</v>
+        <v>654</v>
       </c>
       <c r="AO106" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP106" t="s" s="2">
-        <v>600</v>
+        <v>80</v>
       </c>
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -15414,23 +15379,21 @@
         <v>80</v>
       </c>
       <c r="J107" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>602</v>
+        <v>656</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>603</v>
+        <v>657</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>604</v>
+        <v>658</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O107" t="s" s="2">
-        <v>606</v>
-      </c>
+        <v>659</v>
+      </c>
+      <c r="O107" s="2"/>
       <c r="P107" t="s" s="2">
         <v>80</v>
       </c>
@@ -15478,7 +15441,7 @@
         <v>80</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>601</v>
+        <v>655</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>78</v>
@@ -15490,7 +15453,7 @@
         <v>103</v>
       </c>
       <c r="AJ107" t="s" s="2">
-        <v>607</v>
+        <v>233</v>
       </c>
       <c r="AK107" t="s" s="2">
         <v>80</v>
@@ -15499,10 +15462,10 @@
         <v>80</v>
       </c>
       <c r="AM107" t="s" s="2">
-        <v>608</v>
+        <v>653</v>
       </c>
       <c r="AN107" t="s" s="2">
-        <v>609</v>
+        <v>660</v>
       </c>
       <c r="AO107" t="s" s="2">
         <v>80</v>
@@ -15513,10 +15476,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -15527,28 +15490,32 @@
         <v>78</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H108" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I108" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J108" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>107</v>
+        <v>591</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>108</v>
+        <v>662</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N108" s="2"/>
-      <c r="O108" s="2"/>
+        <v>662</v>
+      </c>
+      <c r="N108" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="O108" t="s" s="2">
+        <v>664</v>
+      </c>
       <c r="P108" t="s" s="2">
         <v>80</v>
       </c>
@@ -15596,19 +15563,19 @@
         <v>80</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>110</v>
+        <v>661</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH108" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI108" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ108" t="s" s="2">
-        <v>80</v>
+        <v>665</v>
       </c>
       <c r="AK108" t="s" s="2">
         <v>80</v>
@@ -15617,10 +15584,10 @@
         <v>80</v>
       </c>
       <c r="AM108" t="s" s="2">
-        <v>80</v>
+        <v>666</v>
       </c>
       <c r="AN108" t="s" s="2">
-        <v>111</v>
+        <v>667</v>
       </c>
       <c r="AO108" t="s" s="2">
         <v>80</v>
@@ -15631,21 +15598,21 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>611</v>
+        <v>668</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>611</v>
+        <v>668</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E109" s="2"/>
       <c r="F109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H109" t="s" s="2">
         <v>80</v>
@@ -15657,17 +15624,15 @@
         <v>80</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N109" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N109" s="2"/>
       <c r="O109" s="2"/>
       <c r="P109" t="s" s="2">
         <v>80</v>
@@ -15704,31 +15669,31 @@
         <v>80</v>
       </c>
       <c r="AB109" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC109" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD109" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE109" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH109" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI109" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ109" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK109" t="s" s="2">
         <v>80</v>
@@ -15740,7 +15705,7 @@
         <v>80</v>
       </c>
       <c r="AN109" t="s" s="2">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="AO109" t="s" s="2">
         <v>80</v>
@@ -15751,14 +15716,14 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>612</v>
+        <v>669</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>612</v>
+        <v>669</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
-        <v>613</v>
+        <v>113</v>
       </c>
       <c r="E110" s="2"/>
       <c r="F110" t="s" s="2">
@@ -15771,26 +15736,24 @@
         <v>80</v>
       </c>
       <c r="I110" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J110" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K110" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>614</v>
+        <v>115</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>615</v>
+        <v>116</v>
       </c>
       <c r="N110" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O110" t="s" s="2">
-        <v>215</v>
-      </c>
+      <c r="O110" s="2"/>
       <c r="P110" t="s" s="2">
         <v>80</v>
       </c>
@@ -15826,19 +15789,19 @@
         <v>80</v>
       </c>
       <c r="AB110" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC110" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE110" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>616</v>
+        <v>121</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>78</v>
@@ -15873,44 +15836,46 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>617</v>
+        <v>670</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>617</v>
+        <v>670</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
-        <v>80</v>
+        <v>602</v>
       </c>
       <c r="E111" s="2"/>
       <c r="F111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G111" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H111" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I111" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J111" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>618</v>
+        <v>114</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>619</v>
+        <v>603</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>620</v>
+        <v>604</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="O111" s="2"/>
+        <v>117</v>
+      </c>
+      <c r="O111" t="s" s="2">
+        <v>215</v>
+      </c>
       <c r="P111" t="s" s="2">
         <v>80</v>
       </c>
@@ -15958,19 +15923,19 @@
         <v>80</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH111" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI111" t="s" s="2">
-        <v>622</v>
+        <v>103</v>
       </c>
       <c r="AJ111" t="s" s="2">
-        <v>623</v>
+        <v>122</v>
       </c>
       <c r="AK111" t="s" s="2">
         <v>80</v>
@@ -15979,10 +15944,10 @@
         <v>80</v>
       </c>
       <c r="AM111" t="s" s="2">
-        <v>624</v>
+        <v>80</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>625</v>
+        <v>105</v>
       </c>
       <c r="AO111" t="s" s="2">
         <v>80</v>
@@ -15993,10 +15958,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -16004,33 +15969,35 @@
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H112" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J112" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>618</v>
+        <v>260</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>627</v>
+        <v>672</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>628</v>
+        <v>673</v>
       </c>
       <c r="N112" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="O112" s="2"/>
+        <v>674</v>
+      </c>
+      <c r="O112" t="s" s="2">
+        <v>675</v>
+      </c>
       <c r="P112" t="s" s="2">
         <v>80</v>
       </c>
@@ -16054,13 +16021,13 @@
         <v>80</v>
       </c>
       <c r="X112" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="Y112" t="s" s="2">
-        <v>80</v>
+        <v>351</v>
       </c>
       <c r="Z112" t="s" s="2">
-        <v>80</v>
+        <v>352</v>
       </c>
       <c r="AA112" t="s" s="2">
         <v>80</v>
@@ -16078,34 +16045,34 @@
         <v>80</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>626</v>
+        <v>671</v>
       </c>
       <c r="AG112" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="AH112" t="s" s="2">
         <v>91</v>
       </c>
       <c r="AI112" t="s" s="2">
-        <v>622</v>
+        <v>103</v>
       </c>
       <c r="AJ112" t="s" s="2">
-        <v>623</v>
+        <v>104</v>
       </c>
       <c r="AK112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>80</v>
+        <v>676</v>
       </c>
       <c r="AM112" t="s" s="2">
-        <v>624</v>
+        <v>355</v>
       </c>
       <c r="AN112" t="s" s="2">
-        <v>629</v>
+        <v>356</v>
       </c>
       <c r="AO112" t="s" s="2">
-        <v>80</v>
+        <v>357</v>
       </c>
       <c r="AP112" t="s" s="2">
         <v>80</v>
@@ -16113,10 +16080,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -16130,28 +16097,28 @@
         <v>91</v>
       </c>
       <c r="H113" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J113" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>260</v>
+        <v>678</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>631</v>
+        <v>679</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>632</v>
+        <v>680</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>633</v>
+        <v>681</v>
       </c>
       <c r="O113" t="s" s="2">
-        <v>634</v>
+        <v>442</v>
       </c>
       <c r="P113" t="s" s="2">
         <v>80</v>
@@ -16176,13 +16143,13 @@
         <v>80</v>
       </c>
       <c r="X113" t="s" s="2">
-        <v>175</v>
+        <v>251</v>
       </c>
       <c r="Y113" t="s" s="2">
-        <v>635</v>
+        <v>682</v>
       </c>
       <c r="Z113" t="s" s="2">
-        <v>636</v>
+        <v>683</v>
       </c>
       <c r="AA113" t="s" s="2">
         <v>80</v>
@@ -16200,7 +16167,7 @@
         <v>80</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>630</v>
+        <v>677</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
@@ -16209,7 +16176,7 @@
         <v>91</v>
       </c>
       <c r="AI113" t="s" s="2">
-        <v>103</v>
+        <v>684</v>
       </c>
       <c r="AJ113" t="s" s="2">
         <v>104</v>
@@ -16218,27 +16185,27 @@
         <v>80</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>637</v>
+        <v>685</v>
       </c>
       <c r="AM113" t="s" s="2">
-        <v>638</v>
+        <v>447</v>
       </c>
       <c r="AN113" t="s" s="2">
-        <v>534</v>
+        <v>448</v>
       </c>
       <c r="AO113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP113" t="s" s="2">
-        <v>80</v>
+        <v>449</v>
       </c>
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -16249,10 +16216,10 @@
         <v>78</v>
       </c>
       <c r="G114" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H114" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I114" t="s" s="2">
         <v>80</v>
@@ -16264,16 +16231,16 @@
         <v>260</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>640</v>
+        <v>687</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>641</v>
+        <v>688</v>
       </c>
       <c r="N114" t="s" s="2">
-        <v>642</v>
+        <v>689</v>
       </c>
       <c r="O114" t="s" s="2">
-        <v>643</v>
+        <v>509</v>
       </c>
       <c r="P114" t="s" s="2">
         <v>80</v>
@@ -16298,13 +16265,13 @@
         <v>80</v>
       </c>
       <c r="X114" t="s" s="2">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="Y114" t="s" s="2">
-        <v>644</v>
+        <v>510</v>
       </c>
       <c r="Z114" t="s" s="2">
-        <v>645</v>
+        <v>511</v>
       </c>
       <c r="AA114" t="s" s="2">
         <v>80</v>
@@ -16322,16 +16289,16 @@
         <v>80</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>639</v>
+        <v>686</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH114" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI114" t="s" s="2">
-        <v>103</v>
+        <v>690</v>
       </c>
       <c r="AJ114" t="s" s="2">
         <v>104</v>
@@ -16340,13 +16307,13 @@
         <v>80</v>
       </c>
       <c r="AL114" t="s" s="2">
-        <v>637</v>
+        <v>80</v>
       </c>
       <c r="AM114" t="s" s="2">
-        <v>638</v>
+        <v>105</v>
       </c>
       <c r="AN114" t="s" s="2">
-        <v>534</v>
+        <v>513</v>
       </c>
       <c r="AO114" t="s" s="2">
         <v>80</v>
@@ -16357,21 +16324,21 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
-        <v>80</v>
+        <v>526</v>
       </c>
       <c r="E115" s="2"/>
       <c r="F115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G115" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H115" t="s" s="2">
         <v>80</v>
@@ -16383,19 +16350,19 @@
         <v>80</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>647</v>
+        <v>260</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>648</v>
+        <v>527</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>649</v>
+        <v>528</v>
       </c>
       <c r="N115" t="s" s="2">
-        <v>650</v>
+        <v>529</v>
       </c>
       <c r="O115" t="s" s="2">
-        <v>651</v>
+        <v>530</v>
       </c>
       <c r="P115" t="s" s="2">
         <v>80</v>
@@ -16420,13 +16387,13 @@
         <v>80</v>
       </c>
       <c r="X115" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="Y115" t="s" s="2">
-        <v>80</v>
+        <v>692</v>
       </c>
       <c r="Z115" t="s" s="2">
-        <v>80</v>
+        <v>531</v>
       </c>
       <c r="AA115" t="s" s="2">
         <v>80</v>
@@ -16444,45 +16411,45 @@
         <v>80</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>646</v>
+        <v>691</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH115" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI115" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ115" t="s" s="2">
-        <v>652</v>
+        <v>104</v>
       </c>
       <c r="AK115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>80</v>
+        <v>532</v>
       </c>
       <c r="AM115" t="s" s="2">
-        <v>653</v>
+        <v>533</v>
       </c>
       <c r="AN115" t="s" s="2">
-        <v>654</v>
+        <v>534</v>
       </c>
       <c r="AO115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP115" t="s" s="2">
-        <v>80</v>
+        <v>535</v>
       </c>
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -16493,7 +16460,7 @@
         <v>78</v>
       </c>
       <c r="G116" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H116" t="s" s="2">
         <v>80</v>
@@ -16505,18 +16472,20 @@
         <v>80</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>656</v>
+        <v>694</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>657</v>
+        <v>695</v>
       </c>
       <c r="N116" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="O116" s="2"/>
+        <v>594</v>
+      </c>
+      <c r="O116" t="s" s="2">
+        <v>595</v>
+      </c>
       <c r="P116" t="s" s="2">
         <v>80</v>
       </c>
@@ -16564,19 +16533,19 @@
         <v>80</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>655</v>
+        <v>693</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH116" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI116" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ116" t="s" s="2">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="AK116" t="s" s="2">
         <v>80</v>
@@ -16585,1352 +16554,20 @@
         <v>80</v>
       </c>
       <c r="AM116" t="s" s="2">
-        <v>624</v>
+        <v>597</v>
       </c>
       <c r="AN116" t="s" s="2">
-        <v>658</v>
+        <v>598</v>
       </c>
       <c r="AO116" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP116" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="117" hidden="true">
-      <c r="A117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="B117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="C117" s="2"/>
-      <c r="D117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E117" s="2"/>
-      <c r="F117" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G117" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J117" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K117" t="s" s="2">
-        <v>660</v>
-      </c>
-      <c r="L117" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="M117" t="s" s="2">
-        <v>662</v>
-      </c>
-      <c r="N117" t="s" s="2">
-        <v>663</v>
-      </c>
-      <c r="O117" s="2"/>
-      <c r="P117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q117" s="2"/>
-      <c r="R117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF117" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="AG117" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH117" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI117" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ117" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="AK117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM117" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="AN117" t="s" s="2">
-        <v>665</v>
-      </c>
-      <c r="AO117" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP117" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="118" hidden="true">
-      <c r="A118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="B118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="C118" s="2"/>
-      <c r="D118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E118" s="2"/>
-      <c r="F118" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G118" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J118" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K118" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="L118" t="s" s="2">
-        <v>668</v>
-      </c>
-      <c r="M118" t="s" s="2">
-        <v>669</v>
-      </c>
-      <c r="N118" t="s" s="2">
-        <v>670</v>
-      </c>
-      <c r="O118" s="2"/>
-      <c r="P118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q118" s="2"/>
-      <c r="R118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF118" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="AG118" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH118" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI118" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ118" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="AK118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM118" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="AN118" t="s" s="2">
-        <v>671</v>
-      </c>
-      <c r="AO118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP118" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="119" hidden="true">
-      <c r="A119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="B119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="C119" s="2"/>
-      <c r="D119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E119" s="2"/>
-      <c r="F119" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G119" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H119" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J119" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K119" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="L119" t="s" s="2">
-        <v>673</v>
-      </c>
-      <c r="M119" t="s" s="2">
-        <v>673</v>
-      </c>
-      <c r="N119" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="O119" t="s" s="2">
-        <v>675</v>
-      </c>
-      <c r="P119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q119" s="2"/>
-      <c r="R119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF119" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="AG119" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH119" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI119" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ119" t="s" s="2">
-        <v>676</v>
-      </c>
-      <c r="AK119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM119" t="s" s="2">
-        <v>677</v>
-      </c>
-      <c r="AN119" t="s" s="2">
-        <v>678</v>
-      </c>
-      <c r="AO119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP119" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="120" hidden="true">
-      <c r="A120" t="s" s="2">
-        <v>679</v>
-      </c>
-      <c r="B120" t="s" s="2">
-        <v>679</v>
-      </c>
-      <c r="C120" s="2"/>
-      <c r="D120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E120" s="2"/>
-      <c r="F120" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G120" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K120" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="L120" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N120" s="2"/>
-      <c r="O120" s="2"/>
-      <c r="P120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q120" s="2"/>
-      <c r="R120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF120" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="AG120" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH120" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN120" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="AO120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP120" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="121" hidden="true">
-      <c r="A121" t="s" s="2">
-        <v>680</v>
-      </c>
-      <c r="B121" t="s" s="2">
-        <v>680</v>
-      </c>
-      <c r="C121" s="2"/>
-      <c r="D121" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="E121" s="2"/>
-      <c r="F121" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G121" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K121" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="L121" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="M121" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N121" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O121" s="2"/>
-      <c r="P121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q121" s="2"/>
-      <c r="R121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB121" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AC121" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="AD121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE121" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="AF121" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="AG121" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH121" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI121" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ121" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="AK121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN121" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AO121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP121" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="122" hidden="true">
-      <c r="A122" t="s" s="2">
-        <v>681</v>
-      </c>
-      <c r="B122" t="s" s="2">
-        <v>681</v>
-      </c>
-      <c r="C122" s="2"/>
-      <c r="D122" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="E122" s="2"/>
-      <c r="F122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G122" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I122" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="J122" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K122" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="L122" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>615</v>
-      </c>
-      <c r="N122" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O122" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="P122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q122" s="2"/>
-      <c r="R122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF122" t="s" s="2">
-        <v>616</v>
-      </c>
-      <c r="AG122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH122" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI122" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ122" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="AK122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN122" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AO122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP122" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="123" hidden="true">
-      <c r="A123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="B123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="C123" s="2"/>
-      <c r="D123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E123" s="2"/>
-      <c r="F123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="G123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H123" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J123" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K123" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L123" t="s" s="2">
-        <v>683</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>684</v>
-      </c>
-      <c r="N123" t="s" s="2">
-        <v>685</v>
-      </c>
-      <c r="O123" t="s" s="2">
-        <v>686</v>
-      </c>
-      <c r="P123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q123" s="2"/>
-      <c r="R123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X123" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y123" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="Z123" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="AA123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF123" t="s" s="2">
-        <v>682</v>
-      </c>
-      <c r="AG123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AH123" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI123" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ123" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL123" t="s" s="2">
-        <v>687</v>
-      </c>
-      <c r="AM123" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="AN123" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="AO123" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="AP123" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="124" hidden="true">
-      <c r="A124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="B124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="C124" s="2"/>
-      <c r="D124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E124" s="2"/>
-      <c r="F124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G124" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H124" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J124" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="K124" t="s" s="2">
-        <v>689</v>
-      </c>
-      <c r="L124" t="s" s="2">
-        <v>690</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>691</v>
-      </c>
-      <c r="N124" t="s" s="2">
-        <v>692</v>
-      </c>
-      <c r="O124" t="s" s="2">
-        <v>442</v>
-      </c>
-      <c r="P124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q124" s="2"/>
-      <c r="R124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X124" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="Y124" t="s" s="2">
-        <v>693</v>
-      </c>
-      <c r="Z124" t="s" s="2">
-        <v>694</v>
-      </c>
-      <c r="AA124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF124" t="s" s="2">
-        <v>688</v>
-      </c>
-      <c r="AG124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH124" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI124" t="s" s="2">
-        <v>695</v>
-      </c>
-      <c r="AJ124" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL124" t="s" s="2">
-        <v>696</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="AN124" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="AO124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP124" t="s" s="2">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="125" hidden="true">
-      <c r="A125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="B125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="C125" s="2"/>
-      <c r="D125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E125" s="2"/>
-      <c r="F125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G125" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="H125" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="I125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K125" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L125" t="s" s="2">
-        <v>698</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>699</v>
-      </c>
-      <c r="N125" t="s" s="2">
-        <v>700</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>509</v>
-      </c>
-      <c r="P125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q125" s="2"/>
-      <c r="R125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X125" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y125" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="Z125" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="AA125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF125" t="s" s="2">
-        <v>697</v>
-      </c>
-      <c r="AG125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH125" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AI125" t="s" s="2">
-        <v>701</v>
-      </c>
-      <c r="AJ125" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AN125" t="s" s="2">
-        <v>513</v>
-      </c>
-      <c r="AO125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP125" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="126" hidden="true">
-      <c r="A126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="B126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="C126" s="2"/>
-      <c r="D126" t="s" s="2">
-        <v>526</v>
-      </c>
-      <c r="E126" s="2"/>
-      <c r="F126" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G126" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K126" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L126" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>528</v>
-      </c>
-      <c r="N126" t="s" s="2">
-        <v>529</v>
-      </c>
-      <c r="O126" t="s" s="2">
-        <v>530</v>
-      </c>
-      <c r="P126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q126" s="2"/>
-      <c r="R126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X126" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="Y126" t="s" s="2">
-        <v>703</v>
-      </c>
-      <c r="Z126" t="s" s="2">
-        <v>531</v>
-      </c>
-      <c r="AA126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF126" t="s" s="2">
-        <v>702</v>
-      </c>
-      <c r="AG126" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH126" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI126" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="AJ126" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="AK126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL126" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="AM126" t="s" s="2">
-        <v>533</v>
-      </c>
-      <c r="AN126" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="AO126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP126" t="s" s="2">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="127" hidden="true">
-      <c r="A127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="B127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="C127" s="2"/>
-      <c r="D127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E127" s="2"/>
-      <c r="F127" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G127" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K127" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="L127" t="s" s="2">
-        <v>705</v>
-      </c>
-      <c r="M127" t="s" s="2">
-        <v>706</v>
-      </c>
-      <c r="N127" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O127" t="s" s="2">
-        <v>606</v>
-      </c>
-      <c r="P127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q127" s="2"/>
-      <c r="R127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF127" t="s" s="2">
-        <v>704</v>
-      </c>
-      <c r="AG127" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH127" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM127" t="s" s="2">
-        <v>608</v>
-      </c>
-      <c r="AN127" t="s" s="2">
-        <v>609</v>
-      </c>
-      <c r="AO127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP127" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP127">
+  <autoFilter ref="A1:AP116">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -17940,7 +16577,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI126">
+  <conditionalFormatting sqref="A2:AI115">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>